<commit_message>
Full customer addresses, and franchises trade as Robocode <place>
Addresses: customers gain address1/address2/city/postcode/country. schema.sql
adds them with add-column-if-not-exists and folds the old single-line address
into address1 before dropping it, so it applies to the live database as it
stands. The Customers tab now has the fields, every row has an Edit button that
loads the record back into the form, and the table shows the address so gaps are
obvious. The bulk-import template and parser carry the same columns.

Naming: a franchise is stored as the place name alone and displayed as
'Robocode Shirley' by a single custLabel helper, used in the orders list, order
detail, money owed, balances, pickers, CSV exports and the invoice. It will not
double the prefix if someone types it in anyway. Schools and individuals are
untouched.

Invoices now print the full multi-line address in the Invoice to block, and the
filename and title use the trading name.
</commit_message>
<xml_diff>
--- a/templates/customers.xlsx
+++ b/templates/customers.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G303"/>
+  <dimension ref="A1:K303"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -505,8 +505,12 @@
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -519,7 +523,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>One row per customer, starting on row 4. Upload this file on the Customers tab of the app. Only "name" and "type" are required. Do not rename or reorder the headers. See the Example tab for how it should look.</t>
+          <t>One row per customer, starting on row 4. Upload this file on the Customers tab of the app. Only "name" and "type" are required, but the address is what prints on invoices. For a franchise put just the place name - invoices add the "Robocode" prefix. Do not rename or reorder the headers. See the Example tab.</t>
         </is>
       </c>
     </row>
@@ -551,10 +555,30 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>address</t>
+          <t>address1</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>address2</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>city</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>postcode</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -568,6 +592,10 @@
       <c r="E4" s="4" t="n"/>
       <c r="F4" s="4" t="n"/>
       <c r="G4" s="4" t="n"/>
+      <c r="H4" s="4" t="n"/>
+      <c r="I4" s="4" t="n"/>
+      <c r="J4" s="4" t="n"/>
+      <c r="K4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n"/>
@@ -577,6 +605,10 @@
       <c r="E5" s="4" t="n"/>
       <c r="F5" s="4" t="n"/>
       <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="n"/>
+      <c r="I5" s="4" t="n"/>
+      <c r="J5" s="4" t="n"/>
+      <c r="K5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n"/>
@@ -586,6 +618,10 @@
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="4" t="n"/>
       <c r="G6" s="4" t="n"/>
+      <c r="H6" s="4" t="n"/>
+      <c r="I6" s="4" t="n"/>
+      <c r="J6" s="4" t="n"/>
+      <c r="K6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n"/>
@@ -595,6 +631,10 @@
       <c r="E7" s="4" t="n"/>
       <c r="F7" s="4" t="n"/>
       <c r="G7" s="4" t="n"/>
+      <c r="H7" s="4" t="n"/>
+      <c r="I7" s="4" t="n"/>
+      <c r="J7" s="4" t="n"/>
+      <c r="K7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n"/>
@@ -604,6 +644,10 @@
       <c r="E8" s="4" t="n"/>
       <c r="F8" s="4" t="n"/>
       <c r="G8" s="4" t="n"/>
+      <c r="H8" s="4" t="n"/>
+      <c r="I8" s="4" t="n"/>
+      <c r="J8" s="4" t="n"/>
+      <c r="K8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n"/>
@@ -613,6 +657,10 @@
       <c r="E9" s="4" t="n"/>
       <c r="F9" s="4" t="n"/>
       <c r="G9" s="4" t="n"/>
+      <c r="H9" s="4" t="n"/>
+      <c r="I9" s="4" t="n"/>
+      <c r="J9" s="4" t="n"/>
+      <c r="K9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n"/>
@@ -622,6 +670,10 @@
       <c r="E10" s="4" t="n"/>
       <c r="F10" s="4" t="n"/>
       <c r="G10" s="4" t="n"/>
+      <c r="H10" s="4" t="n"/>
+      <c r="I10" s="4" t="n"/>
+      <c r="J10" s="4" t="n"/>
+      <c r="K10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n"/>
@@ -631,6 +683,10 @@
       <c r="E11" s="4" t="n"/>
       <c r="F11" s="4" t="n"/>
       <c r="G11" s="4" t="n"/>
+      <c r="H11" s="4" t="n"/>
+      <c r="I11" s="4" t="n"/>
+      <c r="J11" s="4" t="n"/>
+      <c r="K11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n"/>
@@ -640,6 +696,10 @@
       <c r="E12" s="4" t="n"/>
       <c r="F12" s="4" t="n"/>
       <c r="G12" s="4" t="n"/>
+      <c r="H12" s="4" t="n"/>
+      <c r="I12" s="4" t="n"/>
+      <c r="J12" s="4" t="n"/>
+      <c r="K12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n"/>
@@ -649,6 +709,10 @@
       <c r="E13" s="4" t="n"/>
       <c r="F13" s="4" t="n"/>
       <c r="G13" s="4" t="n"/>
+      <c r="H13" s="4" t="n"/>
+      <c r="I13" s="4" t="n"/>
+      <c r="J13" s="4" t="n"/>
+      <c r="K13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n"/>
@@ -658,6 +722,10 @@
       <c r="E14" s="4" t="n"/>
       <c r="F14" s="4" t="n"/>
       <c r="G14" s="4" t="n"/>
+      <c r="H14" s="4" t="n"/>
+      <c r="I14" s="4" t="n"/>
+      <c r="J14" s="4" t="n"/>
+      <c r="K14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n"/>
@@ -667,6 +735,10 @@
       <c r="E15" s="4" t="n"/>
       <c r="F15" s="4" t="n"/>
       <c r="G15" s="4" t="n"/>
+      <c r="H15" s="4" t="n"/>
+      <c r="I15" s="4" t="n"/>
+      <c r="J15" s="4" t="n"/>
+      <c r="K15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n"/>
@@ -676,6 +748,10 @@
       <c r="E16" s="4" t="n"/>
       <c r="F16" s="4" t="n"/>
       <c r="G16" s="4" t="n"/>
+      <c r="H16" s="4" t="n"/>
+      <c r="I16" s="4" t="n"/>
+      <c r="J16" s="4" t="n"/>
+      <c r="K16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n"/>
@@ -685,6 +761,10 @@
       <c r="E17" s="4" t="n"/>
       <c r="F17" s="4" t="n"/>
       <c r="G17" s="4" t="n"/>
+      <c r="H17" s="4" t="n"/>
+      <c r="I17" s="4" t="n"/>
+      <c r="J17" s="4" t="n"/>
+      <c r="K17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n"/>
@@ -694,6 +774,10 @@
       <c r="E18" s="4" t="n"/>
       <c r="F18" s="4" t="n"/>
       <c r="G18" s="4" t="n"/>
+      <c r="H18" s="4" t="n"/>
+      <c r="I18" s="4" t="n"/>
+      <c r="J18" s="4" t="n"/>
+      <c r="K18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n"/>
@@ -703,6 +787,10 @@
       <c r="E19" s="4" t="n"/>
       <c r="F19" s="4" t="n"/>
       <c r="G19" s="4" t="n"/>
+      <c r="H19" s="4" t="n"/>
+      <c r="I19" s="4" t="n"/>
+      <c r="J19" s="4" t="n"/>
+      <c r="K19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n"/>
@@ -712,6 +800,10 @@
       <c r="E20" s="4" t="n"/>
       <c r="F20" s="4" t="n"/>
       <c r="G20" s="4" t="n"/>
+      <c r="H20" s="4" t="n"/>
+      <c r="I20" s="4" t="n"/>
+      <c r="J20" s="4" t="n"/>
+      <c r="K20" s="4" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n"/>
@@ -721,6 +813,10 @@
       <c r="E21" s="4" t="n"/>
       <c r="F21" s="4" t="n"/>
       <c r="G21" s="4" t="n"/>
+      <c r="H21" s="4" t="n"/>
+      <c r="I21" s="4" t="n"/>
+      <c r="J21" s="4" t="n"/>
+      <c r="K21" s="4" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n"/>
@@ -730,6 +826,10 @@
       <c r="E22" s="4" t="n"/>
       <c r="F22" s="4" t="n"/>
       <c r="G22" s="4" t="n"/>
+      <c r="H22" s="4" t="n"/>
+      <c r="I22" s="4" t="n"/>
+      <c r="J22" s="4" t="n"/>
+      <c r="K22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n"/>
@@ -739,6 +839,10 @@
       <c r="E23" s="4" t="n"/>
       <c r="F23" s="4" t="n"/>
       <c r="G23" s="4" t="n"/>
+      <c r="H23" s="4" t="n"/>
+      <c r="I23" s="4" t="n"/>
+      <c r="J23" s="4" t="n"/>
+      <c r="K23" s="4" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n"/>
@@ -748,6 +852,10 @@
       <c r="E24" s="4" t="n"/>
       <c r="F24" s="4" t="n"/>
       <c r="G24" s="4" t="n"/>
+      <c r="H24" s="4" t="n"/>
+      <c r="I24" s="4" t="n"/>
+      <c r="J24" s="4" t="n"/>
+      <c r="K24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n"/>
@@ -757,6 +865,10 @@
       <c r="E25" s="4" t="n"/>
       <c r="F25" s="4" t="n"/>
       <c r="G25" s="4" t="n"/>
+      <c r="H25" s="4" t="n"/>
+      <c r="I25" s="4" t="n"/>
+      <c r="J25" s="4" t="n"/>
+      <c r="K25" s="4" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n"/>
@@ -766,6 +878,10 @@
       <c r="E26" s="4" t="n"/>
       <c r="F26" s="4" t="n"/>
       <c r="G26" s="4" t="n"/>
+      <c r="H26" s="4" t="n"/>
+      <c r="I26" s="4" t="n"/>
+      <c r="J26" s="4" t="n"/>
+      <c r="K26" s="4" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n"/>
@@ -775,6 +891,10 @@
       <c r="E27" s="4" t="n"/>
       <c r="F27" s="4" t="n"/>
       <c r="G27" s="4" t="n"/>
+      <c r="H27" s="4" t="n"/>
+      <c r="I27" s="4" t="n"/>
+      <c r="J27" s="4" t="n"/>
+      <c r="K27" s="4" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n"/>
@@ -784,6 +904,10 @@
       <c r="E28" s="4" t="n"/>
       <c r="F28" s="4" t="n"/>
       <c r="G28" s="4" t="n"/>
+      <c r="H28" s="4" t="n"/>
+      <c r="I28" s="4" t="n"/>
+      <c r="J28" s="4" t="n"/>
+      <c r="K28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n"/>
@@ -793,6 +917,10 @@
       <c r="E29" s="4" t="n"/>
       <c r="F29" s="4" t="n"/>
       <c r="G29" s="4" t="n"/>
+      <c r="H29" s="4" t="n"/>
+      <c r="I29" s="4" t="n"/>
+      <c r="J29" s="4" t="n"/>
+      <c r="K29" s="4" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n"/>
@@ -802,6 +930,10 @@
       <c r="E30" s="4" t="n"/>
       <c r="F30" s="4" t="n"/>
       <c r="G30" s="4" t="n"/>
+      <c r="H30" s="4" t="n"/>
+      <c r="I30" s="4" t="n"/>
+      <c r="J30" s="4" t="n"/>
+      <c r="K30" s="4" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n"/>
@@ -811,6 +943,10 @@
       <c r="E31" s="4" t="n"/>
       <c r="F31" s="4" t="n"/>
       <c r="G31" s="4" t="n"/>
+      <c r="H31" s="4" t="n"/>
+      <c r="I31" s="4" t="n"/>
+      <c r="J31" s="4" t="n"/>
+      <c r="K31" s="4" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n"/>
@@ -820,6 +956,10 @@
       <c r="E32" s="4" t="n"/>
       <c r="F32" s="4" t="n"/>
       <c r="G32" s="4" t="n"/>
+      <c r="H32" s="4" t="n"/>
+      <c r="I32" s="4" t="n"/>
+      <c r="J32" s="4" t="n"/>
+      <c r="K32" s="4" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n"/>
@@ -829,6 +969,10 @@
       <c r="E33" s="4" t="n"/>
       <c r="F33" s="4" t="n"/>
       <c r="G33" s="4" t="n"/>
+      <c r="H33" s="4" t="n"/>
+      <c r="I33" s="4" t="n"/>
+      <c r="J33" s="4" t="n"/>
+      <c r="K33" s="4" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n"/>
@@ -838,6 +982,10 @@
       <c r="E34" s="4" t="n"/>
       <c r="F34" s="4" t="n"/>
       <c r="G34" s="4" t="n"/>
+      <c r="H34" s="4" t="n"/>
+      <c r="I34" s="4" t="n"/>
+      <c r="J34" s="4" t="n"/>
+      <c r="K34" s="4" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n"/>
@@ -847,6 +995,10 @@
       <c r="E35" s="4" t="n"/>
       <c r="F35" s="4" t="n"/>
       <c r="G35" s="4" t="n"/>
+      <c r="H35" s="4" t="n"/>
+      <c r="I35" s="4" t="n"/>
+      <c r="J35" s="4" t="n"/>
+      <c r="K35" s="4" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n"/>
@@ -856,6 +1008,10 @@
       <c r="E36" s="4" t="n"/>
       <c r="F36" s="4" t="n"/>
       <c r="G36" s="4" t="n"/>
+      <c r="H36" s="4" t="n"/>
+      <c r="I36" s="4" t="n"/>
+      <c r="J36" s="4" t="n"/>
+      <c r="K36" s="4" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n"/>
@@ -865,6 +1021,10 @@
       <c r="E37" s="4" t="n"/>
       <c r="F37" s="4" t="n"/>
       <c r="G37" s="4" t="n"/>
+      <c r="H37" s="4" t="n"/>
+      <c r="I37" s="4" t="n"/>
+      <c r="J37" s="4" t="n"/>
+      <c r="K37" s="4" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n"/>
@@ -874,6 +1034,10 @@
       <c r="E38" s="4" t="n"/>
       <c r="F38" s="4" t="n"/>
       <c r="G38" s="4" t="n"/>
+      <c r="H38" s="4" t="n"/>
+      <c r="I38" s="4" t="n"/>
+      <c r="J38" s="4" t="n"/>
+      <c r="K38" s="4" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n"/>
@@ -883,6 +1047,10 @@
       <c r="E39" s="4" t="n"/>
       <c r="F39" s="4" t="n"/>
       <c r="G39" s="4" t="n"/>
+      <c r="H39" s="4" t="n"/>
+      <c r="I39" s="4" t="n"/>
+      <c r="J39" s="4" t="n"/>
+      <c r="K39" s="4" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="n"/>
@@ -892,6 +1060,10 @@
       <c r="E40" s="4" t="n"/>
       <c r="F40" s="4" t="n"/>
       <c r="G40" s="4" t="n"/>
+      <c r="H40" s="4" t="n"/>
+      <c r="I40" s="4" t="n"/>
+      <c r="J40" s="4" t="n"/>
+      <c r="K40" s="4" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n"/>
@@ -901,6 +1073,10 @@
       <c r="E41" s="4" t="n"/>
       <c r="F41" s="4" t="n"/>
       <c r="G41" s="4" t="n"/>
+      <c r="H41" s="4" t="n"/>
+      <c r="I41" s="4" t="n"/>
+      <c r="J41" s="4" t="n"/>
+      <c r="K41" s="4" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="n"/>
@@ -910,6 +1086,10 @@
       <c r="E42" s="4" t="n"/>
       <c r="F42" s="4" t="n"/>
       <c r="G42" s="4" t="n"/>
+      <c r="H42" s="4" t="n"/>
+      <c r="I42" s="4" t="n"/>
+      <c r="J42" s="4" t="n"/>
+      <c r="K42" s="4" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="n"/>
@@ -919,6 +1099,10 @@
       <c r="E43" s="4" t="n"/>
       <c r="F43" s="4" t="n"/>
       <c r="G43" s="4" t="n"/>
+      <c r="H43" s="4" t="n"/>
+      <c r="I43" s="4" t="n"/>
+      <c r="J43" s="4" t="n"/>
+      <c r="K43" s="4" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="n"/>
@@ -928,6 +1112,10 @@
       <c r="E44" s="4" t="n"/>
       <c r="F44" s="4" t="n"/>
       <c r="G44" s="4" t="n"/>
+      <c r="H44" s="4" t="n"/>
+      <c r="I44" s="4" t="n"/>
+      <c r="J44" s="4" t="n"/>
+      <c r="K44" s="4" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n"/>
@@ -937,6 +1125,10 @@
       <c r="E45" s="4" t="n"/>
       <c r="F45" s="4" t="n"/>
       <c r="G45" s="4" t="n"/>
+      <c r="H45" s="4" t="n"/>
+      <c r="I45" s="4" t="n"/>
+      <c r="J45" s="4" t="n"/>
+      <c r="K45" s="4" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="n"/>
@@ -946,6 +1138,10 @@
       <c r="E46" s="4" t="n"/>
       <c r="F46" s="4" t="n"/>
       <c r="G46" s="4" t="n"/>
+      <c r="H46" s="4" t="n"/>
+      <c r="I46" s="4" t="n"/>
+      <c r="J46" s="4" t="n"/>
+      <c r="K46" s="4" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n"/>
@@ -955,6 +1151,10 @@
       <c r="E47" s="4" t="n"/>
       <c r="F47" s="4" t="n"/>
       <c r="G47" s="4" t="n"/>
+      <c r="H47" s="4" t="n"/>
+      <c r="I47" s="4" t="n"/>
+      <c r="J47" s="4" t="n"/>
+      <c r="K47" s="4" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="n"/>
@@ -964,6 +1164,10 @@
       <c r="E48" s="4" t="n"/>
       <c r="F48" s="4" t="n"/>
       <c r="G48" s="4" t="n"/>
+      <c r="H48" s="4" t="n"/>
+      <c r="I48" s="4" t="n"/>
+      <c r="J48" s="4" t="n"/>
+      <c r="K48" s="4" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="n"/>
@@ -973,6 +1177,10 @@
       <c r="E49" s="4" t="n"/>
       <c r="F49" s="4" t="n"/>
       <c r="G49" s="4" t="n"/>
+      <c r="H49" s="4" t="n"/>
+      <c r="I49" s="4" t="n"/>
+      <c r="J49" s="4" t="n"/>
+      <c r="K49" s="4" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="4" t="n"/>
@@ -982,6 +1190,10 @@
       <c r="E50" s="4" t="n"/>
       <c r="F50" s="4" t="n"/>
       <c r="G50" s="4" t="n"/>
+      <c r="H50" s="4" t="n"/>
+      <c r="I50" s="4" t="n"/>
+      <c r="J50" s="4" t="n"/>
+      <c r="K50" s="4" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="n"/>
@@ -991,6 +1203,10 @@
       <c r="E51" s="4" t="n"/>
       <c r="F51" s="4" t="n"/>
       <c r="G51" s="4" t="n"/>
+      <c r="H51" s="4" t="n"/>
+      <c r="I51" s="4" t="n"/>
+      <c r="J51" s="4" t="n"/>
+      <c r="K51" s="4" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="n"/>
@@ -1000,6 +1216,10 @@
       <c r="E52" s="4" t="n"/>
       <c r="F52" s="4" t="n"/>
       <c r="G52" s="4" t="n"/>
+      <c r="H52" s="4" t="n"/>
+      <c r="I52" s="4" t="n"/>
+      <c r="J52" s="4" t="n"/>
+      <c r="K52" s="4" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="4" t="n"/>
@@ -1009,6 +1229,10 @@
       <c r="E53" s="4" t="n"/>
       <c r="F53" s="4" t="n"/>
       <c r="G53" s="4" t="n"/>
+      <c r="H53" s="4" t="n"/>
+      <c r="I53" s="4" t="n"/>
+      <c r="J53" s="4" t="n"/>
+      <c r="K53" s="4" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="n"/>
@@ -1018,6 +1242,10 @@
       <c r="E54" s="4" t="n"/>
       <c r="F54" s="4" t="n"/>
       <c r="G54" s="4" t="n"/>
+      <c r="H54" s="4" t="n"/>
+      <c r="I54" s="4" t="n"/>
+      <c r="J54" s="4" t="n"/>
+      <c r="K54" s="4" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="4" t="n"/>
@@ -1027,6 +1255,10 @@
       <c r="E55" s="4" t="n"/>
       <c r="F55" s="4" t="n"/>
       <c r="G55" s="4" t="n"/>
+      <c r="H55" s="4" t="n"/>
+      <c r="I55" s="4" t="n"/>
+      <c r="J55" s="4" t="n"/>
+      <c r="K55" s="4" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="4" t="n"/>
@@ -1036,6 +1268,10 @@
       <c r="E56" s="4" t="n"/>
       <c r="F56" s="4" t="n"/>
       <c r="G56" s="4" t="n"/>
+      <c r="H56" s="4" t="n"/>
+      <c r="I56" s="4" t="n"/>
+      <c r="J56" s="4" t="n"/>
+      <c r="K56" s="4" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="n"/>
@@ -1045,6 +1281,10 @@
       <c r="E57" s="4" t="n"/>
       <c r="F57" s="4" t="n"/>
       <c r="G57" s="4" t="n"/>
+      <c r="H57" s="4" t="n"/>
+      <c r="I57" s="4" t="n"/>
+      <c r="J57" s="4" t="n"/>
+      <c r="K57" s="4" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="4" t="n"/>
@@ -1054,6 +1294,10 @@
       <c r="E58" s="4" t="n"/>
       <c r="F58" s="4" t="n"/>
       <c r="G58" s="4" t="n"/>
+      <c r="H58" s="4" t="n"/>
+      <c r="I58" s="4" t="n"/>
+      <c r="J58" s="4" t="n"/>
+      <c r="K58" s="4" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="4" t="n"/>
@@ -1063,6 +1307,10 @@
       <c r="E59" s="4" t="n"/>
       <c r="F59" s="4" t="n"/>
       <c r="G59" s="4" t="n"/>
+      <c r="H59" s="4" t="n"/>
+      <c r="I59" s="4" t="n"/>
+      <c r="J59" s="4" t="n"/>
+      <c r="K59" s="4" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="n"/>
@@ -1072,6 +1320,10 @@
       <c r="E60" s="4" t="n"/>
       <c r="F60" s="4" t="n"/>
       <c r="G60" s="4" t="n"/>
+      <c r="H60" s="4" t="n"/>
+      <c r="I60" s="4" t="n"/>
+      <c r="J60" s="4" t="n"/>
+      <c r="K60" s="4" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="n"/>
@@ -1081,6 +1333,10 @@
       <c r="E61" s="4" t="n"/>
       <c r="F61" s="4" t="n"/>
       <c r="G61" s="4" t="n"/>
+      <c r="H61" s="4" t="n"/>
+      <c r="I61" s="4" t="n"/>
+      <c r="J61" s="4" t="n"/>
+      <c r="K61" s="4" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="4" t="n"/>
@@ -1090,6 +1346,10 @@
       <c r="E62" s="4" t="n"/>
       <c r="F62" s="4" t="n"/>
       <c r="G62" s="4" t="n"/>
+      <c r="H62" s="4" t="n"/>
+      <c r="I62" s="4" t="n"/>
+      <c r="J62" s="4" t="n"/>
+      <c r="K62" s="4" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="4" t="n"/>
@@ -1099,6 +1359,10 @@
       <c r="E63" s="4" t="n"/>
       <c r="F63" s="4" t="n"/>
       <c r="G63" s="4" t="n"/>
+      <c r="H63" s="4" t="n"/>
+      <c r="I63" s="4" t="n"/>
+      <c r="J63" s="4" t="n"/>
+      <c r="K63" s="4" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="4" t="n"/>
@@ -1108,6 +1372,10 @@
       <c r="E64" s="4" t="n"/>
       <c r="F64" s="4" t="n"/>
       <c r="G64" s="4" t="n"/>
+      <c r="H64" s="4" t="n"/>
+      <c r="I64" s="4" t="n"/>
+      <c r="J64" s="4" t="n"/>
+      <c r="K64" s="4" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="4" t="n"/>
@@ -1117,6 +1385,10 @@
       <c r="E65" s="4" t="n"/>
       <c r="F65" s="4" t="n"/>
       <c r="G65" s="4" t="n"/>
+      <c r="H65" s="4" t="n"/>
+      <c r="I65" s="4" t="n"/>
+      <c r="J65" s="4" t="n"/>
+      <c r="K65" s="4" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="4" t="n"/>
@@ -1126,6 +1398,10 @@
       <c r="E66" s="4" t="n"/>
       <c r="F66" s="4" t="n"/>
       <c r="G66" s="4" t="n"/>
+      <c r="H66" s="4" t="n"/>
+      <c r="I66" s="4" t="n"/>
+      <c r="J66" s="4" t="n"/>
+      <c r="K66" s="4" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="4" t="n"/>
@@ -1135,6 +1411,10 @@
       <c r="E67" s="4" t="n"/>
       <c r="F67" s="4" t="n"/>
       <c r="G67" s="4" t="n"/>
+      <c r="H67" s="4" t="n"/>
+      <c r="I67" s="4" t="n"/>
+      <c r="J67" s="4" t="n"/>
+      <c r="K67" s="4" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="4" t="n"/>
@@ -1144,6 +1424,10 @@
       <c r="E68" s="4" t="n"/>
       <c r="F68" s="4" t="n"/>
       <c r="G68" s="4" t="n"/>
+      <c r="H68" s="4" t="n"/>
+      <c r="I68" s="4" t="n"/>
+      <c r="J68" s="4" t="n"/>
+      <c r="K68" s="4" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="4" t="n"/>
@@ -1153,6 +1437,10 @@
       <c r="E69" s="4" t="n"/>
       <c r="F69" s="4" t="n"/>
       <c r="G69" s="4" t="n"/>
+      <c r="H69" s="4" t="n"/>
+      <c r="I69" s="4" t="n"/>
+      <c r="J69" s="4" t="n"/>
+      <c r="K69" s="4" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="4" t="n"/>
@@ -1162,6 +1450,10 @@
       <c r="E70" s="4" t="n"/>
       <c r="F70" s="4" t="n"/>
       <c r="G70" s="4" t="n"/>
+      <c r="H70" s="4" t="n"/>
+      <c r="I70" s="4" t="n"/>
+      <c r="J70" s="4" t="n"/>
+      <c r="K70" s="4" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="4" t="n"/>
@@ -1171,6 +1463,10 @@
       <c r="E71" s="4" t="n"/>
       <c r="F71" s="4" t="n"/>
       <c r="G71" s="4" t="n"/>
+      <c r="H71" s="4" t="n"/>
+      <c r="I71" s="4" t="n"/>
+      <c r="J71" s="4" t="n"/>
+      <c r="K71" s="4" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="4" t="n"/>
@@ -1180,6 +1476,10 @@
       <c r="E72" s="4" t="n"/>
       <c r="F72" s="4" t="n"/>
       <c r="G72" s="4" t="n"/>
+      <c r="H72" s="4" t="n"/>
+      <c r="I72" s="4" t="n"/>
+      <c r="J72" s="4" t="n"/>
+      <c r="K72" s="4" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="4" t="n"/>
@@ -1189,6 +1489,10 @@
       <c r="E73" s="4" t="n"/>
       <c r="F73" s="4" t="n"/>
       <c r="G73" s="4" t="n"/>
+      <c r="H73" s="4" t="n"/>
+      <c r="I73" s="4" t="n"/>
+      <c r="J73" s="4" t="n"/>
+      <c r="K73" s="4" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="4" t="n"/>
@@ -1198,6 +1502,10 @@
       <c r="E74" s="4" t="n"/>
       <c r="F74" s="4" t="n"/>
       <c r="G74" s="4" t="n"/>
+      <c r="H74" s="4" t="n"/>
+      <c r="I74" s="4" t="n"/>
+      <c r="J74" s="4" t="n"/>
+      <c r="K74" s="4" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="4" t="n"/>
@@ -1207,6 +1515,10 @@
       <c r="E75" s="4" t="n"/>
       <c r="F75" s="4" t="n"/>
       <c r="G75" s="4" t="n"/>
+      <c r="H75" s="4" t="n"/>
+      <c r="I75" s="4" t="n"/>
+      <c r="J75" s="4" t="n"/>
+      <c r="K75" s="4" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="4" t="n"/>
@@ -1216,6 +1528,10 @@
       <c r="E76" s="4" t="n"/>
       <c r="F76" s="4" t="n"/>
       <c r="G76" s="4" t="n"/>
+      <c r="H76" s="4" t="n"/>
+      <c r="I76" s="4" t="n"/>
+      <c r="J76" s="4" t="n"/>
+      <c r="K76" s="4" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="4" t="n"/>
@@ -1225,6 +1541,10 @@
       <c r="E77" s="4" t="n"/>
       <c r="F77" s="4" t="n"/>
       <c r="G77" s="4" t="n"/>
+      <c r="H77" s="4" t="n"/>
+      <c r="I77" s="4" t="n"/>
+      <c r="J77" s="4" t="n"/>
+      <c r="K77" s="4" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="4" t="n"/>
@@ -1234,6 +1554,10 @@
       <c r="E78" s="4" t="n"/>
       <c r="F78" s="4" t="n"/>
       <c r="G78" s="4" t="n"/>
+      <c r="H78" s="4" t="n"/>
+      <c r="I78" s="4" t="n"/>
+      <c r="J78" s="4" t="n"/>
+      <c r="K78" s="4" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="4" t="n"/>
@@ -1243,6 +1567,10 @@
       <c r="E79" s="4" t="n"/>
       <c r="F79" s="4" t="n"/>
       <c r="G79" s="4" t="n"/>
+      <c r="H79" s="4" t="n"/>
+      <c r="I79" s="4" t="n"/>
+      <c r="J79" s="4" t="n"/>
+      <c r="K79" s="4" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="4" t="n"/>
@@ -1252,6 +1580,10 @@
       <c r="E80" s="4" t="n"/>
       <c r="F80" s="4" t="n"/>
       <c r="G80" s="4" t="n"/>
+      <c r="H80" s="4" t="n"/>
+      <c r="I80" s="4" t="n"/>
+      <c r="J80" s="4" t="n"/>
+      <c r="K80" s="4" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="4" t="n"/>
@@ -1261,6 +1593,10 @@
       <c r="E81" s="4" t="n"/>
       <c r="F81" s="4" t="n"/>
       <c r="G81" s="4" t="n"/>
+      <c r="H81" s="4" t="n"/>
+      <c r="I81" s="4" t="n"/>
+      <c r="J81" s="4" t="n"/>
+      <c r="K81" s="4" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="4" t="n"/>
@@ -1270,6 +1606,10 @@
       <c r="E82" s="4" t="n"/>
       <c r="F82" s="4" t="n"/>
       <c r="G82" s="4" t="n"/>
+      <c r="H82" s="4" t="n"/>
+      <c r="I82" s="4" t="n"/>
+      <c r="J82" s="4" t="n"/>
+      <c r="K82" s="4" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="4" t="n"/>
@@ -1279,6 +1619,10 @@
       <c r="E83" s="4" t="n"/>
       <c r="F83" s="4" t="n"/>
       <c r="G83" s="4" t="n"/>
+      <c r="H83" s="4" t="n"/>
+      <c r="I83" s="4" t="n"/>
+      <c r="J83" s="4" t="n"/>
+      <c r="K83" s="4" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="4" t="n"/>
@@ -1288,6 +1632,10 @@
       <c r="E84" s="4" t="n"/>
       <c r="F84" s="4" t="n"/>
       <c r="G84" s="4" t="n"/>
+      <c r="H84" s="4" t="n"/>
+      <c r="I84" s="4" t="n"/>
+      <c r="J84" s="4" t="n"/>
+      <c r="K84" s="4" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="4" t="n"/>
@@ -1297,6 +1645,10 @@
       <c r="E85" s="4" t="n"/>
       <c r="F85" s="4" t="n"/>
       <c r="G85" s="4" t="n"/>
+      <c r="H85" s="4" t="n"/>
+      <c r="I85" s="4" t="n"/>
+      <c r="J85" s="4" t="n"/>
+      <c r="K85" s="4" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="4" t="n"/>
@@ -1306,6 +1658,10 @@
       <c r="E86" s="4" t="n"/>
       <c r="F86" s="4" t="n"/>
       <c r="G86" s="4" t="n"/>
+      <c r="H86" s="4" t="n"/>
+      <c r="I86" s="4" t="n"/>
+      <c r="J86" s="4" t="n"/>
+      <c r="K86" s="4" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="4" t="n"/>
@@ -1315,6 +1671,10 @@
       <c r="E87" s="4" t="n"/>
       <c r="F87" s="4" t="n"/>
       <c r="G87" s="4" t="n"/>
+      <c r="H87" s="4" t="n"/>
+      <c r="I87" s="4" t="n"/>
+      <c r="J87" s="4" t="n"/>
+      <c r="K87" s="4" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="4" t="n"/>
@@ -1324,6 +1684,10 @@
       <c r="E88" s="4" t="n"/>
       <c r="F88" s="4" t="n"/>
       <c r="G88" s="4" t="n"/>
+      <c r="H88" s="4" t="n"/>
+      <c r="I88" s="4" t="n"/>
+      <c r="J88" s="4" t="n"/>
+      <c r="K88" s="4" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="4" t="n"/>
@@ -1333,6 +1697,10 @@
       <c r="E89" s="4" t="n"/>
       <c r="F89" s="4" t="n"/>
       <c r="G89" s="4" t="n"/>
+      <c r="H89" s="4" t="n"/>
+      <c r="I89" s="4" t="n"/>
+      <c r="J89" s="4" t="n"/>
+      <c r="K89" s="4" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="4" t="n"/>
@@ -1342,6 +1710,10 @@
       <c r="E90" s="4" t="n"/>
       <c r="F90" s="4" t="n"/>
       <c r="G90" s="4" t="n"/>
+      <c r="H90" s="4" t="n"/>
+      <c r="I90" s="4" t="n"/>
+      <c r="J90" s="4" t="n"/>
+      <c r="K90" s="4" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="4" t="n"/>
@@ -1351,6 +1723,10 @@
       <c r="E91" s="4" t="n"/>
       <c r="F91" s="4" t="n"/>
       <c r="G91" s="4" t="n"/>
+      <c r="H91" s="4" t="n"/>
+      <c r="I91" s="4" t="n"/>
+      <c r="J91" s="4" t="n"/>
+      <c r="K91" s="4" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="4" t="n"/>
@@ -1360,6 +1736,10 @@
       <c r="E92" s="4" t="n"/>
       <c r="F92" s="4" t="n"/>
       <c r="G92" s="4" t="n"/>
+      <c r="H92" s="4" t="n"/>
+      <c r="I92" s="4" t="n"/>
+      <c r="J92" s="4" t="n"/>
+      <c r="K92" s="4" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="4" t="n"/>
@@ -1369,6 +1749,10 @@
       <c r="E93" s="4" t="n"/>
       <c r="F93" s="4" t="n"/>
       <c r="G93" s="4" t="n"/>
+      <c r="H93" s="4" t="n"/>
+      <c r="I93" s="4" t="n"/>
+      <c r="J93" s="4" t="n"/>
+      <c r="K93" s="4" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="4" t="n"/>
@@ -1378,6 +1762,10 @@
       <c r="E94" s="4" t="n"/>
       <c r="F94" s="4" t="n"/>
       <c r="G94" s="4" t="n"/>
+      <c r="H94" s="4" t="n"/>
+      <c r="I94" s="4" t="n"/>
+      <c r="J94" s="4" t="n"/>
+      <c r="K94" s="4" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="4" t="n"/>
@@ -1387,6 +1775,10 @@
       <c r="E95" s="4" t="n"/>
       <c r="F95" s="4" t="n"/>
       <c r="G95" s="4" t="n"/>
+      <c r="H95" s="4" t="n"/>
+      <c r="I95" s="4" t="n"/>
+      <c r="J95" s="4" t="n"/>
+      <c r="K95" s="4" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="4" t="n"/>
@@ -1396,6 +1788,10 @@
       <c r="E96" s="4" t="n"/>
       <c r="F96" s="4" t="n"/>
       <c r="G96" s="4" t="n"/>
+      <c r="H96" s="4" t="n"/>
+      <c r="I96" s="4" t="n"/>
+      <c r="J96" s="4" t="n"/>
+      <c r="K96" s="4" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="4" t="n"/>
@@ -1405,6 +1801,10 @@
       <c r="E97" s="4" t="n"/>
       <c r="F97" s="4" t="n"/>
       <c r="G97" s="4" t="n"/>
+      <c r="H97" s="4" t="n"/>
+      <c r="I97" s="4" t="n"/>
+      <c r="J97" s="4" t="n"/>
+      <c r="K97" s="4" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="4" t="n"/>
@@ -1414,6 +1814,10 @@
       <c r="E98" s="4" t="n"/>
       <c r="F98" s="4" t="n"/>
       <c r="G98" s="4" t="n"/>
+      <c r="H98" s="4" t="n"/>
+      <c r="I98" s="4" t="n"/>
+      <c r="J98" s="4" t="n"/>
+      <c r="K98" s="4" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="4" t="n"/>
@@ -1423,6 +1827,10 @@
       <c r="E99" s="4" t="n"/>
       <c r="F99" s="4" t="n"/>
       <c r="G99" s="4" t="n"/>
+      <c r="H99" s="4" t="n"/>
+      <c r="I99" s="4" t="n"/>
+      <c r="J99" s="4" t="n"/>
+      <c r="K99" s="4" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="4" t="n"/>
@@ -1432,6 +1840,10 @@
       <c r="E100" s="4" t="n"/>
       <c r="F100" s="4" t="n"/>
       <c r="G100" s="4" t="n"/>
+      <c r="H100" s="4" t="n"/>
+      <c r="I100" s="4" t="n"/>
+      <c r="J100" s="4" t="n"/>
+      <c r="K100" s="4" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="4" t="n"/>
@@ -1441,6 +1853,10 @@
       <c r="E101" s="4" t="n"/>
       <c r="F101" s="4" t="n"/>
       <c r="G101" s="4" t="n"/>
+      <c r="H101" s="4" t="n"/>
+      <c r="I101" s="4" t="n"/>
+      <c r="J101" s="4" t="n"/>
+      <c r="K101" s="4" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="4" t="n"/>
@@ -1450,6 +1866,10 @@
       <c r="E102" s="4" t="n"/>
       <c r="F102" s="4" t="n"/>
       <c r="G102" s="4" t="n"/>
+      <c r="H102" s="4" t="n"/>
+      <c r="I102" s="4" t="n"/>
+      <c r="J102" s="4" t="n"/>
+      <c r="K102" s="4" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="4" t="n"/>
@@ -1459,6 +1879,10 @@
       <c r="E103" s="4" t="n"/>
       <c r="F103" s="4" t="n"/>
       <c r="G103" s="4" t="n"/>
+      <c r="H103" s="4" t="n"/>
+      <c r="I103" s="4" t="n"/>
+      <c r="J103" s="4" t="n"/>
+      <c r="K103" s="4" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="4" t="n"/>
@@ -1468,6 +1892,10 @@
       <c r="E104" s="4" t="n"/>
       <c r="F104" s="4" t="n"/>
       <c r="G104" s="4" t="n"/>
+      <c r="H104" s="4" t="n"/>
+      <c r="I104" s="4" t="n"/>
+      <c r="J104" s="4" t="n"/>
+      <c r="K104" s="4" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="4" t="n"/>
@@ -1477,6 +1905,10 @@
       <c r="E105" s="4" t="n"/>
       <c r="F105" s="4" t="n"/>
       <c r="G105" s="4" t="n"/>
+      <c r="H105" s="4" t="n"/>
+      <c r="I105" s="4" t="n"/>
+      <c r="J105" s="4" t="n"/>
+      <c r="K105" s="4" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="4" t="n"/>
@@ -1486,6 +1918,10 @@
       <c r="E106" s="4" t="n"/>
       <c r="F106" s="4" t="n"/>
       <c r="G106" s="4" t="n"/>
+      <c r="H106" s="4" t="n"/>
+      <c r="I106" s="4" t="n"/>
+      <c r="J106" s="4" t="n"/>
+      <c r="K106" s="4" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="4" t="n"/>
@@ -1495,6 +1931,10 @@
       <c r="E107" s="4" t="n"/>
       <c r="F107" s="4" t="n"/>
       <c r="G107" s="4" t="n"/>
+      <c r="H107" s="4" t="n"/>
+      <c r="I107" s="4" t="n"/>
+      <c r="J107" s="4" t="n"/>
+      <c r="K107" s="4" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="4" t="n"/>
@@ -1504,6 +1944,10 @@
       <c r="E108" s="4" t="n"/>
       <c r="F108" s="4" t="n"/>
       <c r="G108" s="4" t="n"/>
+      <c r="H108" s="4" t="n"/>
+      <c r="I108" s="4" t="n"/>
+      <c r="J108" s="4" t="n"/>
+      <c r="K108" s="4" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="4" t="n"/>
@@ -1513,6 +1957,10 @@
       <c r="E109" s="4" t="n"/>
       <c r="F109" s="4" t="n"/>
       <c r="G109" s="4" t="n"/>
+      <c r="H109" s="4" t="n"/>
+      <c r="I109" s="4" t="n"/>
+      <c r="J109" s="4" t="n"/>
+      <c r="K109" s="4" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="4" t="n"/>
@@ -1522,6 +1970,10 @@
       <c r="E110" s="4" t="n"/>
       <c r="F110" s="4" t="n"/>
       <c r="G110" s="4" t="n"/>
+      <c r="H110" s="4" t="n"/>
+      <c r="I110" s="4" t="n"/>
+      <c r="J110" s="4" t="n"/>
+      <c r="K110" s="4" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="4" t="n"/>
@@ -1531,6 +1983,10 @@
       <c r="E111" s="4" t="n"/>
       <c r="F111" s="4" t="n"/>
       <c r="G111" s="4" t="n"/>
+      <c r="H111" s="4" t="n"/>
+      <c r="I111" s="4" t="n"/>
+      <c r="J111" s="4" t="n"/>
+      <c r="K111" s="4" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="4" t="n"/>
@@ -1540,6 +1996,10 @@
       <c r="E112" s="4" t="n"/>
       <c r="F112" s="4" t="n"/>
       <c r="G112" s="4" t="n"/>
+      <c r="H112" s="4" t="n"/>
+      <c r="I112" s="4" t="n"/>
+      <c r="J112" s="4" t="n"/>
+      <c r="K112" s="4" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="4" t="n"/>
@@ -1549,6 +2009,10 @@
       <c r="E113" s="4" t="n"/>
       <c r="F113" s="4" t="n"/>
       <c r="G113" s="4" t="n"/>
+      <c r="H113" s="4" t="n"/>
+      <c r="I113" s="4" t="n"/>
+      <c r="J113" s="4" t="n"/>
+      <c r="K113" s="4" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="4" t="n"/>
@@ -1558,6 +2022,10 @@
       <c r="E114" s="4" t="n"/>
       <c r="F114" s="4" t="n"/>
       <c r="G114" s="4" t="n"/>
+      <c r="H114" s="4" t="n"/>
+      <c r="I114" s="4" t="n"/>
+      <c r="J114" s="4" t="n"/>
+      <c r="K114" s="4" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="4" t="n"/>
@@ -1567,6 +2035,10 @@
       <c r="E115" s="4" t="n"/>
       <c r="F115" s="4" t="n"/>
       <c r="G115" s="4" t="n"/>
+      <c r="H115" s="4" t="n"/>
+      <c r="I115" s="4" t="n"/>
+      <c r="J115" s="4" t="n"/>
+      <c r="K115" s="4" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="4" t="n"/>
@@ -1576,6 +2048,10 @@
       <c r="E116" s="4" t="n"/>
       <c r="F116" s="4" t="n"/>
       <c r="G116" s="4" t="n"/>
+      <c r="H116" s="4" t="n"/>
+      <c r="I116" s="4" t="n"/>
+      <c r="J116" s="4" t="n"/>
+      <c r="K116" s="4" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="4" t="n"/>
@@ -1585,6 +2061,10 @@
       <c r="E117" s="4" t="n"/>
       <c r="F117" s="4" t="n"/>
       <c r="G117" s="4" t="n"/>
+      <c r="H117" s="4" t="n"/>
+      <c r="I117" s="4" t="n"/>
+      <c r="J117" s="4" t="n"/>
+      <c r="K117" s="4" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="4" t="n"/>
@@ -1594,6 +2074,10 @@
       <c r="E118" s="4" t="n"/>
       <c r="F118" s="4" t="n"/>
       <c r="G118" s="4" t="n"/>
+      <c r="H118" s="4" t="n"/>
+      <c r="I118" s="4" t="n"/>
+      <c r="J118" s="4" t="n"/>
+      <c r="K118" s="4" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="4" t="n"/>
@@ -1603,6 +2087,10 @@
       <c r="E119" s="4" t="n"/>
       <c r="F119" s="4" t="n"/>
       <c r="G119" s="4" t="n"/>
+      <c r="H119" s="4" t="n"/>
+      <c r="I119" s="4" t="n"/>
+      <c r="J119" s="4" t="n"/>
+      <c r="K119" s="4" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="4" t="n"/>
@@ -1612,6 +2100,10 @@
       <c r="E120" s="4" t="n"/>
       <c r="F120" s="4" t="n"/>
       <c r="G120" s="4" t="n"/>
+      <c r="H120" s="4" t="n"/>
+      <c r="I120" s="4" t="n"/>
+      <c r="J120" s="4" t="n"/>
+      <c r="K120" s="4" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="4" t="n"/>
@@ -1621,6 +2113,10 @@
       <c r="E121" s="4" t="n"/>
       <c r="F121" s="4" t="n"/>
       <c r="G121" s="4" t="n"/>
+      <c r="H121" s="4" t="n"/>
+      <c r="I121" s="4" t="n"/>
+      <c r="J121" s="4" t="n"/>
+      <c r="K121" s="4" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="4" t="n"/>
@@ -1630,6 +2126,10 @@
       <c r="E122" s="4" t="n"/>
       <c r="F122" s="4" t="n"/>
       <c r="G122" s="4" t="n"/>
+      <c r="H122" s="4" t="n"/>
+      <c r="I122" s="4" t="n"/>
+      <c r="J122" s="4" t="n"/>
+      <c r="K122" s="4" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="4" t="n"/>
@@ -1639,6 +2139,10 @@
       <c r="E123" s="4" t="n"/>
       <c r="F123" s="4" t="n"/>
       <c r="G123" s="4" t="n"/>
+      <c r="H123" s="4" t="n"/>
+      <c r="I123" s="4" t="n"/>
+      <c r="J123" s="4" t="n"/>
+      <c r="K123" s="4" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="4" t="n"/>
@@ -1648,6 +2152,10 @@
       <c r="E124" s="4" t="n"/>
       <c r="F124" s="4" t="n"/>
       <c r="G124" s="4" t="n"/>
+      <c r="H124" s="4" t="n"/>
+      <c r="I124" s="4" t="n"/>
+      <c r="J124" s="4" t="n"/>
+      <c r="K124" s="4" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="4" t="n"/>
@@ -1657,6 +2165,10 @@
       <c r="E125" s="4" t="n"/>
       <c r="F125" s="4" t="n"/>
       <c r="G125" s="4" t="n"/>
+      <c r="H125" s="4" t="n"/>
+      <c r="I125" s="4" t="n"/>
+      <c r="J125" s="4" t="n"/>
+      <c r="K125" s="4" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="4" t="n"/>
@@ -1666,6 +2178,10 @@
       <c r="E126" s="4" t="n"/>
       <c r="F126" s="4" t="n"/>
       <c r="G126" s="4" t="n"/>
+      <c r="H126" s="4" t="n"/>
+      <c r="I126" s="4" t="n"/>
+      <c r="J126" s="4" t="n"/>
+      <c r="K126" s="4" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="4" t="n"/>
@@ -1675,6 +2191,10 @@
       <c r="E127" s="4" t="n"/>
       <c r="F127" s="4" t="n"/>
       <c r="G127" s="4" t="n"/>
+      <c r="H127" s="4" t="n"/>
+      <c r="I127" s="4" t="n"/>
+      <c r="J127" s="4" t="n"/>
+      <c r="K127" s="4" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="4" t="n"/>
@@ -1684,6 +2204,10 @@
       <c r="E128" s="4" t="n"/>
       <c r="F128" s="4" t="n"/>
       <c r="G128" s="4" t="n"/>
+      <c r="H128" s="4" t="n"/>
+      <c r="I128" s="4" t="n"/>
+      <c r="J128" s="4" t="n"/>
+      <c r="K128" s="4" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="4" t="n"/>
@@ -1693,6 +2217,10 @@
       <c r="E129" s="4" t="n"/>
       <c r="F129" s="4" t="n"/>
       <c r="G129" s="4" t="n"/>
+      <c r="H129" s="4" t="n"/>
+      <c r="I129" s="4" t="n"/>
+      <c r="J129" s="4" t="n"/>
+      <c r="K129" s="4" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="4" t="n"/>
@@ -1702,6 +2230,10 @@
       <c r="E130" s="4" t="n"/>
       <c r="F130" s="4" t="n"/>
       <c r="G130" s="4" t="n"/>
+      <c r="H130" s="4" t="n"/>
+      <c r="I130" s="4" t="n"/>
+      <c r="J130" s="4" t="n"/>
+      <c r="K130" s="4" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="4" t="n"/>
@@ -1711,6 +2243,10 @@
       <c r="E131" s="4" t="n"/>
       <c r="F131" s="4" t="n"/>
       <c r="G131" s="4" t="n"/>
+      <c r="H131" s="4" t="n"/>
+      <c r="I131" s="4" t="n"/>
+      <c r="J131" s="4" t="n"/>
+      <c r="K131" s="4" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="4" t="n"/>
@@ -1720,6 +2256,10 @@
       <c r="E132" s="4" t="n"/>
       <c r="F132" s="4" t="n"/>
       <c r="G132" s="4" t="n"/>
+      <c r="H132" s="4" t="n"/>
+      <c r="I132" s="4" t="n"/>
+      <c r="J132" s="4" t="n"/>
+      <c r="K132" s="4" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="4" t="n"/>
@@ -1729,6 +2269,10 @@
       <c r="E133" s="4" t="n"/>
       <c r="F133" s="4" t="n"/>
       <c r="G133" s="4" t="n"/>
+      <c r="H133" s="4" t="n"/>
+      <c r="I133" s="4" t="n"/>
+      <c r="J133" s="4" t="n"/>
+      <c r="K133" s="4" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="4" t="n"/>
@@ -1738,6 +2282,10 @@
       <c r="E134" s="4" t="n"/>
       <c r="F134" s="4" t="n"/>
       <c r="G134" s="4" t="n"/>
+      <c r="H134" s="4" t="n"/>
+      <c r="I134" s="4" t="n"/>
+      <c r="J134" s="4" t="n"/>
+      <c r="K134" s="4" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="4" t="n"/>
@@ -1747,6 +2295,10 @@
       <c r="E135" s="4" t="n"/>
       <c r="F135" s="4" t="n"/>
       <c r="G135" s="4" t="n"/>
+      <c r="H135" s="4" t="n"/>
+      <c r="I135" s="4" t="n"/>
+      <c r="J135" s="4" t="n"/>
+      <c r="K135" s="4" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="4" t="n"/>
@@ -1756,6 +2308,10 @@
       <c r="E136" s="4" t="n"/>
       <c r="F136" s="4" t="n"/>
       <c r="G136" s="4" t="n"/>
+      <c r="H136" s="4" t="n"/>
+      <c r="I136" s="4" t="n"/>
+      <c r="J136" s="4" t="n"/>
+      <c r="K136" s="4" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="4" t="n"/>
@@ -1765,6 +2321,10 @@
       <c r="E137" s="4" t="n"/>
       <c r="F137" s="4" t="n"/>
       <c r="G137" s="4" t="n"/>
+      <c r="H137" s="4" t="n"/>
+      <c r="I137" s="4" t="n"/>
+      <c r="J137" s="4" t="n"/>
+      <c r="K137" s="4" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="4" t="n"/>
@@ -1774,6 +2334,10 @@
       <c r="E138" s="4" t="n"/>
       <c r="F138" s="4" t="n"/>
       <c r="G138" s="4" t="n"/>
+      <c r="H138" s="4" t="n"/>
+      <c r="I138" s="4" t="n"/>
+      <c r="J138" s="4" t="n"/>
+      <c r="K138" s="4" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="4" t="n"/>
@@ -1783,6 +2347,10 @@
       <c r="E139" s="4" t="n"/>
       <c r="F139" s="4" t="n"/>
       <c r="G139" s="4" t="n"/>
+      <c r="H139" s="4" t="n"/>
+      <c r="I139" s="4" t="n"/>
+      <c r="J139" s="4" t="n"/>
+      <c r="K139" s="4" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="4" t="n"/>
@@ -1792,6 +2360,10 @@
       <c r="E140" s="4" t="n"/>
       <c r="F140" s="4" t="n"/>
       <c r="G140" s="4" t="n"/>
+      <c r="H140" s="4" t="n"/>
+      <c r="I140" s="4" t="n"/>
+      <c r="J140" s="4" t="n"/>
+      <c r="K140" s="4" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="4" t="n"/>
@@ -1801,6 +2373,10 @@
       <c r="E141" s="4" t="n"/>
       <c r="F141" s="4" t="n"/>
       <c r="G141" s="4" t="n"/>
+      <c r="H141" s="4" t="n"/>
+      <c r="I141" s="4" t="n"/>
+      <c r="J141" s="4" t="n"/>
+      <c r="K141" s="4" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="4" t="n"/>
@@ -1810,6 +2386,10 @@
       <c r="E142" s="4" t="n"/>
       <c r="F142" s="4" t="n"/>
       <c r="G142" s="4" t="n"/>
+      <c r="H142" s="4" t="n"/>
+      <c r="I142" s="4" t="n"/>
+      <c r="J142" s="4" t="n"/>
+      <c r="K142" s="4" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="4" t="n"/>
@@ -1819,6 +2399,10 @@
       <c r="E143" s="4" t="n"/>
       <c r="F143" s="4" t="n"/>
       <c r="G143" s="4" t="n"/>
+      <c r="H143" s="4" t="n"/>
+      <c r="I143" s="4" t="n"/>
+      <c r="J143" s="4" t="n"/>
+      <c r="K143" s="4" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="4" t="n"/>
@@ -1828,6 +2412,10 @@
       <c r="E144" s="4" t="n"/>
       <c r="F144" s="4" t="n"/>
       <c r="G144" s="4" t="n"/>
+      <c r="H144" s="4" t="n"/>
+      <c r="I144" s="4" t="n"/>
+      <c r="J144" s="4" t="n"/>
+      <c r="K144" s="4" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="4" t="n"/>
@@ -1837,6 +2425,10 @@
       <c r="E145" s="4" t="n"/>
       <c r="F145" s="4" t="n"/>
       <c r="G145" s="4" t="n"/>
+      <c r="H145" s="4" t="n"/>
+      <c r="I145" s="4" t="n"/>
+      <c r="J145" s="4" t="n"/>
+      <c r="K145" s="4" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="4" t="n"/>
@@ -1846,6 +2438,10 @@
       <c r="E146" s="4" t="n"/>
       <c r="F146" s="4" t="n"/>
       <c r="G146" s="4" t="n"/>
+      <c r="H146" s="4" t="n"/>
+      <c r="I146" s="4" t="n"/>
+      <c r="J146" s="4" t="n"/>
+      <c r="K146" s="4" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="4" t="n"/>
@@ -1855,6 +2451,10 @@
       <c r="E147" s="4" t="n"/>
       <c r="F147" s="4" t="n"/>
       <c r="G147" s="4" t="n"/>
+      <c r="H147" s="4" t="n"/>
+      <c r="I147" s="4" t="n"/>
+      <c r="J147" s="4" t="n"/>
+      <c r="K147" s="4" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="4" t="n"/>
@@ -1864,6 +2464,10 @@
       <c r="E148" s="4" t="n"/>
       <c r="F148" s="4" t="n"/>
       <c r="G148" s="4" t="n"/>
+      <c r="H148" s="4" t="n"/>
+      <c r="I148" s="4" t="n"/>
+      <c r="J148" s="4" t="n"/>
+      <c r="K148" s="4" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="4" t="n"/>
@@ -1873,6 +2477,10 @@
       <c r="E149" s="4" t="n"/>
       <c r="F149" s="4" t="n"/>
       <c r="G149" s="4" t="n"/>
+      <c r="H149" s="4" t="n"/>
+      <c r="I149" s="4" t="n"/>
+      <c r="J149" s="4" t="n"/>
+      <c r="K149" s="4" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="4" t="n"/>
@@ -1882,6 +2490,10 @@
       <c r="E150" s="4" t="n"/>
       <c r="F150" s="4" t="n"/>
       <c r="G150" s="4" t="n"/>
+      <c r="H150" s="4" t="n"/>
+      <c r="I150" s="4" t="n"/>
+      <c r="J150" s="4" t="n"/>
+      <c r="K150" s="4" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="4" t="n"/>
@@ -1891,6 +2503,10 @@
       <c r="E151" s="4" t="n"/>
       <c r="F151" s="4" t="n"/>
       <c r="G151" s="4" t="n"/>
+      <c r="H151" s="4" t="n"/>
+      <c r="I151" s="4" t="n"/>
+      <c r="J151" s="4" t="n"/>
+      <c r="K151" s="4" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="4" t="n"/>
@@ -1900,6 +2516,10 @@
       <c r="E152" s="4" t="n"/>
       <c r="F152" s="4" t="n"/>
       <c r="G152" s="4" t="n"/>
+      <c r="H152" s="4" t="n"/>
+      <c r="I152" s="4" t="n"/>
+      <c r="J152" s="4" t="n"/>
+      <c r="K152" s="4" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="4" t="n"/>
@@ -1909,6 +2529,10 @@
       <c r="E153" s="4" t="n"/>
       <c r="F153" s="4" t="n"/>
       <c r="G153" s="4" t="n"/>
+      <c r="H153" s="4" t="n"/>
+      <c r="I153" s="4" t="n"/>
+      <c r="J153" s="4" t="n"/>
+      <c r="K153" s="4" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="4" t="n"/>
@@ -1918,6 +2542,10 @@
       <c r="E154" s="4" t="n"/>
       <c r="F154" s="4" t="n"/>
       <c r="G154" s="4" t="n"/>
+      <c r="H154" s="4" t="n"/>
+      <c r="I154" s="4" t="n"/>
+      <c r="J154" s="4" t="n"/>
+      <c r="K154" s="4" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="4" t="n"/>
@@ -1927,6 +2555,10 @@
       <c r="E155" s="4" t="n"/>
       <c r="F155" s="4" t="n"/>
       <c r="G155" s="4" t="n"/>
+      <c r="H155" s="4" t="n"/>
+      <c r="I155" s="4" t="n"/>
+      <c r="J155" s="4" t="n"/>
+      <c r="K155" s="4" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="4" t="n"/>
@@ -1936,6 +2568,10 @@
       <c r="E156" s="4" t="n"/>
       <c r="F156" s="4" t="n"/>
       <c r="G156" s="4" t="n"/>
+      <c r="H156" s="4" t="n"/>
+      <c r="I156" s="4" t="n"/>
+      <c r="J156" s="4" t="n"/>
+      <c r="K156" s="4" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="4" t="n"/>
@@ -1945,6 +2581,10 @@
       <c r="E157" s="4" t="n"/>
       <c r="F157" s="4" t="n"/>
       <c r="G157" s="4" t="n"/>
+      <c r="H157" s="4" t="n"/>
+      <c r="I157" s="4" t="n"/>
+      <c r="J157" s="4" t="n"/>
+      <c r="K157" s="4" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="4" t="n"/>
@@ -1954,6 +2594,10 @@
       <c r="E158" s="4" t="n"/>
       <c r="F158" s="4" t="n"/>
       <c r="G158" s="4" t="n"/>
+      <c r="H158" s="4" t="n"/>
+      <c r="I158" s="4" t="n"/>
+      <c r="J158" s="4" t="n"/>
+      <c r="K158" s="4" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="4" t="n"/>
@@ -1963,6 +2607,10 @@
       <c r="E159" s="4" t="n"/>
       <c r="F159" s="4" t="n"/>
       <c r="G159" s="4" t="n"/>
+      <c r="H159" s="4" t="n"/>
+      <c r="I159" s="4" t="n"/>
+      <c r="J159" s="4" t="n"/>
+      <c r="K159" s="4" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="4" t="n"/>
@@ -1972,6 +2620,10 @@
       <c r="E160" s="4" t="n"/>
       <c r="F160" s="4" t="n"/>
       <c r="G160" s="4" t="n"/>
+      <c r="H160" s="4" t="n"/>
+      <c r="I160" s="4" t="n"/>
+      <c r="J160" s="4" t="n"/>
+      <c r="K160" s="4" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="4" t="n"/>
@@ -1981,6 +2633,10 @@
       <c r="E161" s="4" t="n"/>
       <c r="F161" s="4" t="n"/>
       <c r="G161" s="4" t="n"/>
+      <c r="H161" s="4" t="n"/>
+      <c r="I161" s="4" t="n"/>
+      <c r="J161" s="4" t="n"/>
+      <c r="K161" s="4" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="4" t="n"/>
@@ -1990,6 +2646,10 @@
       <c r="E162" s="4" t="n"/>
       <c r="F162" s="4" t="n"/>
       <c r="G162" s="4" t="n"/>
+      <c r="H162" s="4" t="n"/>
+      <c r="I162" s="4" t="n"/>
+      <c r="J162" s="4" t="n"/>
+      <c r="K162" s="4" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="4" t="n"/>
@@ -1999,6 +2659,10 @@
       <c r="E163" s="4" t="n"/>
       <c r="F163" s="4" t="n"/>
       <c r="G163" s="4" t="n"/>
+      <c r="H163" s="4" t="n"/>
+      <c r="I163" s="4" t="n"/>
+      <c r="J163" s="4" t="n"/>
+      <c r="K163" s="4" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="4" t="n"/>
@@ -2008,6 +2672,10 @@
       <c r="E164" s="4" t="n"/>
       <c r="F164" s="4" t="n"/>
       <c r="G164" s="4" t="n"/>
+      <c r="H164" s="4" t="n"/>
+      <c r="I164" s="4" t="n"/>
+      <c r="J164" s="4" t="n"/>
+      <c r="K164" s="4" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="4" t="n"/>
@@ -2017,6 +2685,10 @@
       <c r="E165" s="4" t="n"/>
       <c r="F165" s="4" t="n"/>
       <c r="G165" s="4" t="n"/>
+      <c r="H165" s="4" t="n"/>
+      <c r="I165" s="4" t="n"/>
+      <c r="J165" s="4" t="n"/>
+      <c r="K165" s="4" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="4" t="n"/>
@@ -2026,6 +2698,10 @@
       <c r="E166" s="4" t="n"/>
       <c r="F166" s="4" t="n"/>
       <c r="G166" s="4" t="n"/>
+      <c r="H166" s="4" t="n"/>
+      <c r="I166" s="4" t="n"/>
+      <c r="J166" s="4" t="n"/>
+      <c r="K166" s="4" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="4" t="n"/>
@@ -2035,6 +2711,10 @@
       <c r="E167" s="4" t="n"/>
       <c r="F167" s="4" t="n"/>
       <c r="G167" s="4" t="n"/>
+      <c r="H167" s="4" t="n"/>
+      <c r="I167" s="4" t="n"/>
+      <c r="J167" s="4" t="n"/>
+      <c r="K167" s="4" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="4" t="n"/>
@@ -2044,6 +2724,10 @@
       <c r="E168" s="4" t="n"/>
       <c r="F168" s="4" t="n"/>
       <c r="G168" s="4" t="n"/>
+      <c r="H168" s="4" t="n"/>
+      <c r="I168" s="4" t="n"/>
+      <c r="J168" s="4" t="n"/>
+      <c r="K168" s="4" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="4" t="n"/>
@@ -2053,6 +2737,10 @@
       <c r="E169" s="4" t="n"/>
       <c r="F169" s="4" t="n"/>
       <c r="G169" s="4" t="n"/>
+      <c r="H169" s="4" t="n"/>
+      <c r="I169" s="4" t="n"/>
+      <c r="J169" s="4" t="n"/>
+      <c r="K169" s="4" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="4" t="n"/>
@@ -2062,6 +2750,10 @@
       <c r="E170" s="4" t="n"/>
       <c r="F170" s="4" t="n"/>
       <c r="G170" s="4" t="n"/>
+      <c r="H170" s="4" t="n"/>
+      <c r="I170" s="4" t="n"/>
+      <c r="J170" s="4" t="n"/>
+      <c r="K170" s="4" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="4" t="n"/>
@@ -2071,6 +2763,10 @@
       <c r="E171" s="4" t="n"/>
       <c r="F171" s="4" t="n"/>
       <c r="G171" s="4" t="n"/>
+      <c r="H171" s="4" t="n"/>
+      <c r="I171" s="4" t="n"/>
+      <c r="J171" s="4" t="n"/>
+      <c r="K171" s="4" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="4" t="n"/>
@@ -2080,6 +2776,10 @@
       <c r="E172" s="4" t="n"/>
       <c r="F172" s="4" t="n"/>
       <c r="G172" s="4" t="n"/>
+      <c r="H172" s="4" t="n"/>
+      <c r="I172" s="4" t="n"/>
+      <c r="J172" s="4" t="n"/>
+      <c r="K172" s="4" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="4" t="n"/>
@@ -2089,6 +2789,10 @@
       <c r="E173" s="4" t="n"/>
       <c r="F173" s="4" t="n"/>
       <c r="G173" s="4" t="n"/>
+      <c r="H173" s="4" t="n"/>
+      <c r="I173" s="4" t="n"/>
+      <c r="J173" s="4" t="n"/>
+      <c r="K173" s="4" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="4" t="n"/>
@@ -2098,6 +2802,10 @@
       <c r="E174" s="4" t="n"/>
       <c r="F174" s="4" t="n"/>
       <c r="G174" s="4" t="n"/>
+      <c r="H174" s="4" t="n"/>
+      <c r="I174" s="4" t="n"/>
+      <c r="J174" s="4" t="n"/>
+      <c r="K174" s="4" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="4" t="n"/>
@@ -2107,6 +2815,10 @@
       <c r="E175" s="4" t="n"/>
       <c r="F175" s="4" t="n"/>
       <c r="G175" s="4" t="n"/>
+      <c r="H175" s="4" t="n"/>
+      <c r="I175" s="4" t="n"/>
+      <c r="J175" s="4" t="n"/>
+      <c r="K175" s="4" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="4" t="n"/>
@@ -2116,6 +2828,10 @@
       <c r="E176" s="4" t="n"/>
       <c r="F176" s="4" t="n"/>
       <c r="G176" s="4" t="n"/>
+      <c r="H176" s="4" t="n"/>
+      <c r="I176" s="4" t="n"/>
+      <c r="J176" s="4" t="n"/>
+      <c r="K176" s="4" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="4" t="n"/>
@@ -2125,6 +2841,10 @@
       <c r="E177" s="4" t="n"/>
       <c r="F177" s="4" t="n"/>
       <c r="G177" s="4" t="n"/>
+      <c r="H177" s="4" t="n"/>
+      <c r="I177" s="4" t="n"/>
+      <c r="J177" s="4" t="n"/>
+      <c r="K177" s="4" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="4" t="n"/>
@@ -2134,6 +2854,10 @@
       <c r="E178" s="4" t="n"/>
       <c r="F178" s="4" t="n"/>
       <c r="G178" s="4" t="n"/>
+      <c r="H178" s="4" t="n"/>
+      <c r="I178" s="4" t="n"/>
+      <c r="J178" s="4" t="n"/>
+      <c r="K178" s="4" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="4" t="n"/>
@@ -2143,6 +2867,10 @@
       <c r="E179" s="4" t="n"/>
       <c r="F179" s="4" t="n"/>
       <c r="G179" s="4" t="n"/>
+      <c r="H179" s="4" t="n"/>
+      <c r="I179" s="4" t="n"/>
+      <c r="J179" s="4" t="n"/>
+      <c r="K179" s="4" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="4" t="n"/>
@@ -2152,6 +2880,10 @@
       <c r="E180" s="4" t="n"/>
       <c r="F180" s="4" t="n"/>
       <c r="G180" s="4" t="n"/>
+      <c r="H180" s="4" t="n"/>
+      <c r="I180" s="4" t="n"/>
+      <c r="J180" s="4" t="n"/>
+      <c r="K180" s="4" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="4" t="n"/>
@@ -2161,6 +2893,10 @@
       <c r="E181" s="4" t="n"/>
       <c r="F181" s="4" t="n"/>
       <c r="G181" s="4" t="n"/>
+      <c r="H181" s="4" t="n"/>
+      <c r="I181" s="4" t="n"/>
+      <c r="J181" s="4" t="n"/>
+      <c r="K181" s="4" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="4" t="n"/>
@@ -2170,6 +2906,10 @@
       <c r="E182" s="4" t="n"/>
       <c r="F182" s="4" t="n"/>
       <c r="G182" s="4" t="n"/>
+      <c r="H182" s="4" t="n"/>
+      <c r="I182" s="4" t="n"/>
+      <c r="J182" s="4" t="n"/>
+      <c r="K182" s="4" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="4" t="n"/>
@@ -2179,6 +2919,10 @@
       <c r="E183" s="4" t="n"/>
       <c r="F183" s="4" t="n"/>
       <c r="G183" s="4" t="n"/>
+      <c r="H183" s="4" t="n"/>
+      <c r="I183" s="4" t="n"/>
+      <c r="J183" s="4" t="n"/>
+      <c r="K183" s="4" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="4" t="n"/>
@@ -2188,6 +2932,10 @@
       <c r="E184" s="4" t="n"/>
       <c r="F184" s="4" t="n"/>
       <c r="G184" s="4" t="n"/>
+      <c r="H184" s="4" t="n"/>
+      <c r="I184" s="4" t="n"/>
+      <c r="J184" s="4" t="n"/>
+      <c r="K184" s="4" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="4" t="n"/>
@@ -2197,6 +2945,10 @@
       <c r="E185" s="4" t="n"/>
       <c r="F185" s="4" t="n"/>
       <c r="G185" s="4" t="n"/>
+      <c r="H185" s="4" t="n"/>
+      <c r="I185" s="4" t="n"/>
+      <c r="J185" s="4" t="n"/>
+      <c r="K185" s="4" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="4" t="n"/>
@@ -2206,6 +2958,10 @@
       <c r="E186" s="4" t="n"/>
       <c r="F186" s="4" t="n"/>
       <c r="G186" s="4" t="n"/>
+      <c r="H186" s="4" t="n"/>
+      <c r="I186" s="4" t="n"/>
+      <c r="J186" s="4" t="n"/>
+      <c r="K186" s="4" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="4" t="n"/>
@@ -2215,6 +2971,10 @@
       <c r="E187" s="4" t="n"/>
       <c r="F187" s="4" t="n"/>
       <c r="G187" s="4" t="n"/>
+      <c r="H187" s="4" t="n"/>
+      <c r="I187" s="4" t="n"/>
+      <c r="J187" s="4" t="n"/>
+      <c r="K187" s="4" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="4" t="n"/>
@@ -2224,6 +2984,10 @@
       <c r="E188" s="4" t="n"/>
       <c r="F188" s="4" t="n"/>
       <c r="G188" s="4" t="n"/>
+      <c r="H188" s="4" t="n"/>
+      <c r="I188" s="4" t="n"/>
+      <c r="J188" s="4" t="n"/>
+      <c r="K188" s="4" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="4" t="n"/>
@@ -2233,6 +2997,10 @@
       <c r="E189" s="4" t="n"/>
       <c r="F189" s="4" t="n"/>
       <c r="G189" s="4" t="n"/>
+      <c r="H189" s="4" t="n"/>
+      <c r="I189" s="4" t="n"/>
+      <c r="J189" s="4" t="n"/>
+      <c r="K189" s="4" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="4" t="n"/>
@@ -2242,6 +3010,10 @@
       <c r="E190" s="4" t="n"/>
       <c r="F190" s="4" t="n"/>
       <c r="G190" s="4" t="n"/>
+      <c r="H190" s="4" t="n"/>
+      <c r="I190" s="4" t="n"/>
+      <c r="J190" s="4" t="n"/>
+      <c r="K190" s="4" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="4" t="n"/>
@@ -2251,6 +3023,10 @@
       <c r="E191" s="4" t="n"/>
       <c r="F191" s="4" t="n"/>
       <c r="G191" s="4" t="n"/>
+      <c r="H191" s="4" t="n"/>
+      <c r="I191" s="4" t="n"/>
+      <c r="J191" s="4" t="n"/>
+      <c r="K191" s="4" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="4" t="n"/>
@@ -2260,6 +3036,10 @@
       <c r="E192" s="4" t="n"/>
       <c r="F192" s="4" t="n"/>
       <c r="G192" s="4" t="n"/>
+      <c r="H192" s="4" t="n"/>
+      <c r="I192" s="4" t="n"/>
+      <c r="J192" s="4" t="n"/>
+      <c r="K192" s="4" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="4" t="n"/>
@@ -2269,6 +3049,10 @@
       <c r="E193" s="4" t="n"/>
       <c r="F193" s="4" t="n"/>
       <c r="G193" s="4" t="n"/>
+      <c r="H193" s="4" t="n"/>
+      <c r="I193" s="4" t="n"/>
+      <c r="J193" s="4" t="n"/>
+      <c r="K193" s="4" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="4" t="n"/>
@@ -2278,6 +3062,10 @@
       <c r="E194" s="4" t="n"/>
       <c r="F194" s="4" t="n"/>
       <c r="G194" s="4" t="n"/>
+      <c r="H194" s="4" t="n"/>
+      <c r="I194" s="4" t="n"/>
+      <c r="J194" s="4" t="n"/>
+      <c r="K194" s="4" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="4" t="n"/>
@@ -2287,6 +3075,10 @@
       <c r="E195" s="4" t="n"/>
       <c r="F195" s="4" t="n"/>
       <c r="G195" s="4" t="n"/>
+      <c r="H195" s="4" t="n"/>
+      <c r="I195" s="4" t="n"/>
+      <c r="J195" s="4" t="n"/>
+      <c r="K195" s="4" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="4" t="n"/>
@@ -2296,6 +3088,10 @@
       <c r="E196" s="4" t="n"/>
       <c r="F196" s="4" t="n"/>
       <c r="G196" s="4" t="n"/>
+      <c r="H196" s="4" t="n"/>
+      <c r="I196" s="4" t="n"/>
+      <c r="J196" s="4" t="n"/>
+      <c r="K196" s="4" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="4" t="n"/>
@@ -2305,6 +3101,10 @@
       <c r="E197" s="4" t="n"/>
       <c r="F197" s="4" t="n"/>
       <c r="G197" s="4" t="n"/>
+      <c r="H197" s="4" t="n"/>
+      <c r="I197" s="4" t="n"/>
+      <c r="J197" s="4" t="n"/>
+      <c r="K197" s="4" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="4" t="n"/>
@@ -2314,6 +3114,10 @@
       <c r="E198" s="4" t="n"/>
       <c r="F198" s="4" t="n"/>
       <c r="G198" s="4" t="n"/>
+      <c r="H198" s="4" t="n"/>
+      <c r="I198" s="4" t="n"/>
+      <c r="J198" s="4" t="n"/>
+      <c r="K198" s="4" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="4" t="n"/>
@@ -2323,6 +3127,10 @@
       <c r="E199" s="4" t="n"/>
       <c r="F199" s="4" t="n"/>
       <c r="G199" s="4" t="n"/>
+      <c r="H199" s="4" t="n"/>
+      <c r="I199" s="4" t="n"/>
+      <c r="J199" s="4" t="n"/>
+      <c r="K199" s="4" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="4" t="n"/>
@@ -2332,6 +3140,10 @@
       <c r="E200" s="4" t="n"/>
       <c r="F200" s="4" t="n"/>
       <c r="G200" s="4" t="n"/>
+      <c r="H200" s="4" t="n"/>
+      <c r="I200" s="4" t="n"/>
+      <c r="J200" s="4" t="n"/>
+      <c r="K200" s="4" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="4" t="n"/>
@@ -2341,6 +3153,10 @@
       <c r="E201" s="4" t="n"/>
       <c r="F201" s="4" t="n"/>
       <c r="G201" s="4" t="n"/>
+      <c r="H201" s="4" t="n"/>
+      <c r="I201" s="4" t="n"/>
+      <c r="J201" s="4" t="n"/>
+      <c r="K201" s="4" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="4" t="n"/>
@@ -2350,6 +3166,10 @@
       <c r="E202" s="4" t="n"/>
       <c r="F202" s="4" t="n"/>
       <c r="G202" s="4" t="n"/>
+      <c r="H202" s="4" t="n"/>
+      <c r="I202" s="4" t="n"/>
+      <c r="J202" s="4" t="n"/>
+      <c r="K202" s="4" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="4" t="n"/>
@@ -2359,6 +3179,10 @@
       <c r="E203" s="4" t="n"/>
       <c r="F203" s="4" t="n"/>
       <c r="G203" s="4" t="n"/>
+      <c r="H203" s="4" t="n"/>
+      <c r="I203" s="4" t="n"/>
+      <c r="J203" s="4" t="n"/>
+      <c r="K203" s="4" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="4" t="n"/>
@@ -2368,6 +3192,10 @@
       <c r="E204" s="4" t="n"/>
       <c r="F204" s="4" t="n"/>
       <c r="G204" s="4" t="n"/>
+      <c r="H204" s="4" t="n"/>
+      <c r="I204" s="4" t="n"/>
+      <c r="J204" s="4" t="n"/>
+      <c r="K204" s="4" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="4" t="n"/>
@@ -2377,6 +3205,10 @@
       <c r="E205" s="4" t="n"/>
       <c r="F205" s="4" t="n"/>
       <c r="G205" s="4" t="n"/>
+      <c r="H205" s="4" t="n"/>
+      <c r="I205" s="4" t="n"/>
+      <c r="J205" s="4" t="n"/>
+      <c r="K205" s="4" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="4" t="n"/>
@@ -2386,6 +3218,10 @@
       <c r="E206" s="4" t="n"/>
       <c r="F206" s="4" t="n"/>
       <c r="G206" s="4" t="n"/>
+      <c r="H206" s="4" t="n"/>
+      <c r="I206" s="4" t="n"/>
+      <c r="J206" s="4" t="n"/>
+      <c r="K206" s="4" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="4" t="n"/>
@@ -2395,6 +3231,10 @@
       <c r="E207" s="4" t="n"/>
       <c r="F207" s="4" t="n"/>
       <c r="G207" s="4" t="n"/>
+      <c r="H207" s="4" t="n"/>
+      <c r="I207" s="4" t="n"/>
+      <c r="J207" s="4" t="n"/>
+      <c r="K207" s="4" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="4" t="n"/>
@@ -2404,6 +3244,10 @@
       <c r="E208" s="4" t="n"/>
       <c r="F208" s="4" t="n"/>
       <c r="G208" s="4" t="n"/>
+      <c r="H208" s="4" t="n"/>
+      <c r="I208" s="4" t="n"/>
+      <c r="J208" s="4" t="n"/>
+      <c r="K208" s="4" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="4" t="n"/>
@@ -2413,6 +3257,10 @@
       <c r="E209" s="4" t="n"/>
       <c r="F209" s="4" t="n"/>
       <c r="G209" s="4" t="n"/>
+      <c r="H209" s="4" t="n"/>
+      <c r="I209" s="4" t="n"/>
+      <c r="J209" s="4" t="n"/>
+      <c r="K209" s="4" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="4" t="n"/>
@@ -2422,6 +3270,10 @@
       <c r="E210" s="4" t="n"/>
       <c r="F210" s="4" t="n"/>
       <c r="G210" s="4" t="n"/>
+      <c r="H210" s="4" t="n"/>
+      <c r="I210" s="4" t="n"/>
+      <c r="J210" s="4" t="n"/>
+      <c r="K210" s="4" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="4" t="n"/>
@@ -2431,6 +3283,10 @@
       <c r="E211" s="4" t="n"/>
       <c r="F211" s="4" t="n"/>
       <c r="G211" s="4" t="n"/>
+      <c r="H211" s="4" t="n"/>
+      <c r="I211" s="4" t="n"/>
+      <c r="J211" s="4" t="n"/>
+      <c r="K211" s="4" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="4" t="n"/>
@@ -2440,6 +3296,10 @@
       <c r="E212" s="4" t="n"/>
       <c r="F212" s="4" t="n"/>
       <c r="G212" s="4" t="n"/>
+      <c r="H212" s="4" t="n"/>
+      <c r="I212" s="4" t="n"/>
+      <c r="J212" s="4" t="n"/>
+      <c r="K212" s="4" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="4" t="n"/>
@@ -2449,6 +3309,10 @@
       <c r="E213" s="4" t="n"/>
       <c r="F213" s="4" t="n"/>
       <c r="G213" s="4" t="n"/>
+      <c r="H213" s="4" t="n"/>
+      <c r="I213" s="4" t="n"/>
+      <c r="J213" s="4" t="n"/>
+      <c r="K213" s="4" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="4" t="n"/>
@@ -2458,6 +3322,10 @@
       <c r="E214" s="4" t="n"/>
       <c r="F214" s="4" t="n"/>
       <c r="G214" s="4" t="n"/>
+      <c r="H214" s="4" t="n"/>
+      <c r="I214" s="4" t="n"/>
+      <c r="J214" s="4" t="n"/>
+      <c r="K214" s="4" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="4" t="n"/>
@@ -2467,6 +3335,10 @@
       <c r="E215" s="4" t="n"/>
       <c r="F215" s="4" t="n"/>
       <c r="G215" s="4" t="n"/>
+      <c r="H215" s="4" t="n"/>
+      <c r="I215" s="4" t="n"/>
+      <c r="J215" s="4" t="n"/>
+      <c r="K215" s="4" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="4" t="n"/>
@@ -2476,6 +3348,10 @@
       <c r="E216" s="4" t="n"/>
       <c r="F216" s="4" t="n"/>
       <c r="G216" s="4" t="n"/>
+      <c r="H216" s="4" t="n"/>
+      <c r="I216" s="4" t="n"/>
+      <c r="J216" s="4" t="n"/>
+      <c r="K216" s="4" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="4" t="n"/>
@@ -2485,6 +3361,10 @@
       <c r="E217" s="4" t="n"/>
       <c r="F217" s="4" t="n"/>
       <c r="G217" s="4" t="n"/>
+      <c r="H217" s="4" t="n"/>
+      <c r="I217" s="4" t="n"/>
+      <c r="J217" s="4" t="n"/>
+      <c r="K217" s="4" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="4" t="n"/>
@@ -2494,6 +3374,10 @@
       <c r="E218" s="4" t="n"/>
       <c r="F218" s="4" t="n"/>
       <c r="G218" s="4" t="n"/>
+      <c r="H218" s="4" t="n"/>
+      <c r="I218" s="4" t="n"/>
+      <c r="J218" s="4" t="n"/>
+      <c r="K218" s="4" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="4" t="n"/>
@@ -2503,6 +3387,10 @@
       <c r="E219" s="4" t="n"/>
       <c r="F219" s="4" t="n"/>
       <c r="G219" s="4" t="n"/>
+      <c r="H219" s="4" t="n"/>
+      <c r="I219" s="4" t="n"/>
+      <c r="J219" s="4" t="n"/>
+      <c r="K219" s="4" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="4" t="n"/>
@@ -2512,6 +3400,10 @@
       <c r="E220" s="4" t="n"/>
       <c r="F220" s="4" t="n"/>
       <c r="G220" s="4" t="n"/>
+      <c r="H220" s="4" t="n"/>
+      <c r="I220" s="4" t="n"/>
+      <c r="J220" s="4" t="n"/>
+      <c r="K220" s="4" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="4" t="n"/>
@@ -2521,6 +3413,10 @@
       <c r="E221" s="4" t="n"/>
       <c r="F221" s="4" t="n"/>
       <c r="G221" s="4" t="n"/>
+      <c r="H221" s="4" t="n"/>
+      <c r="I221" s="4" t="n"/>
+      <c r="J221" s="4" t="n"/>
+      <c r="K221" s="4" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="4" t="n"/>
@@ -2530,6 +3426,10 @@
       <c r="E222" s="4" t="n"/>
       <c r="F222" s="4" t="n"/>
       <c r="G222" s="4" t="n"/>
+      <c r="H222" s="4" t="n"/>
+      <c r="I222" s="4" t="n"/>
+      <c r="J222" s="4" t="n"/>
+      <c r="K222" s="4" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="4" t="n"/>
@@ -2539,6 +3439,10 @@
       <c r="E223" s="4" t="n"/>
       <c r="F223" s="4" t="n"/>
       <c r="G223" s="4" t="n"/>
+      <c r="H223" s="4" t="n"/>
+      <c r="I223" s="4" t="n"/>
+      <c r="J223" s="4" t="n"/>
+      <c r="K223" s="4" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="4" t="n"/>
@@ -2548,6 +3452,10 @@
       <c r="E224" s="4" t="n"/>
       <c r="F224" s="4" t="n"/>
       <c r="G224" s="4" t="n"/>
+      <c r="H224" s="4" t="n"/>
+      <c r="I224" s="4" t="n"/>
+      <c r="J224" s="4" t="n"/>
+      <c r="K224" s="4" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="4" t="n"/>
@@ -2557,6 +3465,10 @@
       <c r="E225" s="4" t="n"/>
       <c r="F225" s="4" t="n"/>
       <c r="G225" s="4" t="n"/>
+      <c r="H225" s="4" t="n"/>
+      <c r="I225" s="4" t="n"/>
+      <c r="J225" s="4" t="n"/>
+      <c r="K225" s="4" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="4" t="n"/>
@@ -2566,6 +3478,10 @@
       <c r="E226" s="4" t="n"/>
       <c r="F226" s="4" t="n"/>
       <c r="G226" s="4" t="n"/>
+      <c r="H226" s="4" t="n"/>
+      <c r="I226" s="4" t="n"/>
+      <c r="J226" s="4" t="n"/>
+      <c r="K226" s="4" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="4" t="n"/>
@@ -2575,6 +3491,10 @@
       <c r="E227" s="4" t="n"/>
       <c r="F227" s="4" t="n"/>
       <c r="G227" s="4" t="n"/>
+      <c r="H227" s="4" t="n"/>
+      <c r="I227" s="4" t="n"/>
+      <c r="J227" s="4" t="n"/>
+      <c r="K227" s="4" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="4" t="n"/>
@@ -2584,6 +3504,10 @@
       <c r="E228" s="4" t="n"/>
       <c r="F228" s="4" t="n"/>
       <c r="G228" s="4" t="n"/>
+      <c r="H228" s="4" t="n"/>
+      <c r="I228" s="4" t="n"/>
+      <c r="J228" s="4" t="n"/>
+      <c r="K228" s="4" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="4" t="n"/>
@@ -2593,6 +3517,10 @@
       <c r="E229" s="4" t="n"/>
       <c r="F229" s="4" t="n"/>
       <c r="G229" s="4" t="n"/>
+      <c r="H229" s="4" t="n"/>
+      <c r="I229" s="4" t="n"/>
+      <c r="J229" s="4" t="n"/>
+      <c r="K229" s="4" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="4" t="n"/>
@@ -2602,6 +3530,10 @@
       <c r="E230" s="4" t="n"/>
       <c r="F230" s="4" t="n"/>
       <c r="G230" s="4" t="n"/>
+      <c r="H230" s="4" t="n"/>
+      <c r="I230" s="4" t="n"/>
+      <c r="J230" s="4" t="n"/>
+      <c r="K230" s="4" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="4" t="n"/>
@@ -2611,6 +3543,10 @@
       <c r="E231" s="4" t="n"/>
       <c r="F231" s="4" t="n"/>
       <c r="G231" s="4" t="n"/>
+      <c r="H231" s="4" t="n"/>
+      <c r="I231" s="4" t="n"/>
+      <c r="J231" s="4" t="n"/>
+      <c r="K231" s="4" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="4" t="n"/>
@@ -2620,6 +3556,10 @@
       <c r="E232" s="4" t="n"/>
       <c r="F232" s="4" t="n"/>
       <c r="G232" s="4" t="n"/>
+      <c r="H232" s="4" t="n"/>
+      <c r="I232" s="4" t="n"/>
+      <c r="J232" s="4" t="n"/>
+      <c r="K232" s="4" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="4" t="n"/>
@@ -2629,6 +3569,10 @@
       <c r="E233" s="4" t="n"/>
       <c r="F233" s="4" t="n"/>
       <c r="G233" s="4" t="n"/>
+      <c r="H233" s="4" t="n"/>
+      <c r="I233" s="4" t="n"/>
+      <c r="J233" s="4" t="n"/>
+      <c r="K233" s="4" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="4" t="n"/>
@@ -2638,6 +3582,10 @@
       <c r="E234" s="4" t="n"/>
       <c r="F234" s="4" t="n"/>
       <c r="G234" s="4" t="n"/>
+      <c r="H234" s="4" t="n"/>
+      <c r="I234" s="4" t="n"/>
+      <c r="J234" s="4" t="n"/>
+      <c r="K234" s="4" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="4" t="n"/>
@@ -2647,6 +3595,10 @@
       <c r="E235" s="4" t="n"/>
       <c r="F235" s="4" t="n"/>
       <c r="G235" s="4" t="n"/>
+      <c r="H235" s="4" t="n"/>
+      <c r="I235" s="4" t="n"/>
+      <c r="J235" s="4" t="n"/>
+      <c r="K235" s="4" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="4" t="n"/>
@@ -2656,6 +3608,10 @@
       <c r="E236" s="4" t="n"/>
       <c r="F236" s="4" t="n"/>
       <c r="G236" s="4" t="n"/>
+      <c r="H236" s="4" t="n"/>
+      <c r="I236" s="4" t="n"/>
+      <c r="J236" s="4" t="n"/>
+      <c r="K236" s="4" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="4" t="n"/>
@@ -2665,6 +3621,10 @@
       <c r="E237" s="4" t="n"/>
       <c r="F237" s="4" t="n"/>
       <c r="G237" s="4" t="n"/>
+      <c r="H237" s="4" t="n"/>
+      <c r="I237" s="4" t="n"/>
+      <c r="J237" s="4" t="n"/>
+      <c r="K237" s="4" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="4" t="n"/>
@@ -2674,6 +3634,10 @@
       <c r="E238" s="4" t="n"/>
       <c r="F238" s="4" t="n"/>
       <c r="G238" s="4" t="n"/>
+      <c r="H238" s="4" t="n"/>
+      <c r="I238" s="4" t="n"/>
+      <c r="J238" s="4" t="n"/>
+      <c r="K238" s="4" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="4" t="n"/>
@@ -2683,6 +3647,10 @@
       <c r="E239" s="4" t="n"/>
       <c r="F239" s="4" t="n"/>
       <c r="G239" s="4" t="n"/>
+      <c r="H239" s="4" t="n"/>
+      <c r="I239" s="4" t="n"/>
+      <c r="J239" s="4" t="n"/>
+      <c r="K239" s="4" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="4" t="n"/>
@@ -2692,6 +3660,10 @@
       <c r="E240" s="4" t="n"/>
       <c r="F240" s="4" t="n"/>
       <c r="G240" s="4" t="n"/>
+      <c r="H240" s="4" t="n"/>
+      <c r="I240" s="4" t="n"/>
+      <c r="J240" s="4" t="n"/>
+      <c r="K240" s="4" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="4" t="n"/>
@@ -2701,6 +3673,10 @@
       <c r="E241" s="4" t="n"/>
       <c r="F241" s="4" t="n"/>
       <c r="G241" s="4" t="n"/>
+      <c r="H241" s="4" t="n"/>
+      <c r="I241" s="4" t="n"/>
+      <c r="J241" s="4" t="n"/>
+      <c r="K241" s="4" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="4" t="n"/>
@@ -2710,6 +3686,10 @@
       <c r="E242" s="4" t="n"/>
       <c r="F242" s="4" t="n"/>
       <c r="G242" s="4" t="n"/>
+      <c r="H242" s="4" t="n"/>
+      <c r="I242" s="4" t="n"/>
+      <c r="J242" s="4" t="n"/>
+      <c r="K242" s="4" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="4" t="n"/>
@@ -2719,6 +3699,10 @@
       <c r="E243" s="4" t="n"/>
       <c r="F243" s="4" t="n"/>
       <c r="G243" s="4" t="n"/>
+      <c r="H243" s="4" t="n"/>
+      <c r="I243" s="4" t="n"/>
+      <c r="J243" s="4" t="n"/>
+      <c r="K243" s="4" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="4" t="n"/>
@@ -2728,6 +3712,10 @@
       <c r="E244" s="4" t="n"/>
       <c r="F244" s="4" t="n"/>
       <c r="G244" s="4" t="n"/>
+      <c r="H244" s="4" t="n"/>
+      <c r="I244" s="4" t="n"/>
+      <c r="J244" s="4" t="n"/>
+      <c r="K244" s="4" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="4" t="n"/>
@@ -2737,6 +3725,10 @@
       <c r="E245" s="4" t="n"/>
       <c r="F245" s="4" t="n"/>
       <c r="G245" s="4" t="n"/>
+      <c r="H245" s="4" t="n"/>
+      <c r="I245" s="4" t="n"/>
+      <c r="J245" s="4" t="n"/>
+      <c r="K245" s="4" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="4" t="n"/>
@@ -2746,6 +3738,10 @@
       <c r="E246" s="4" t="n"/>
       <c r="F246" s="4" t="n"/>
       <c r="G246" s="4" t="n"/>
+      <c r="H246" s="4" t="n"/>
+      <c r="I246" s="4" t="n"/>
+      <c r="J246" s="4" t="n"/>
+      <c r="K246" s="4" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="4" t="n"/>
@@ -2755,6 +3751,10 @@
       <c r="E247" s="4" t="n"/>
       <c r="F247" s="4" t="n"/>
       <c r="G247" s="4" t="n"/>
+      <c r="H247" s="4" t="n"/>
+      <c r="I247" s="4" t="n"/>
+      <c r="J247" s="4" t="n"/>
+      <c r="K247" s="4" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="4" t="n"/>
@@ -2764,6 +3764,10 @@
       <c r="E248" s="4" t="n"/>
       <c r="F248" s="4" t="n"/>
       <c r="G248" s="4" t="n"/>
+      <c r="H248" s="4" t="n"/>
+      <c r="I248" s="4" t="n"/>
+      <c r="J248" s="4" t="n"/>
+      <c r="K248" s="4" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="4" t="n"/>
@@ -2773,6 +3777,10 @@
       <c r="E249" s="4" t="n"/>
       <c r="F249" s="4" t="n"/>
       <c r="G249" s="4" t="n"/>
+      <c r="H249" s="4" t="n"/>
+      <c r="I249" s="4" t="n"/>
+      <c r="J249" s="4" t="n"/>
+      <c r="K249" s="4" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="4" t="n"/>
@@ -2782,6 +3790,10 @@
       <c r="E250" s="4" t="n"/>
       <c r="F250" s="4" t="n"/>
       <c r="G250" s="4" t="n"/>
+      <c r="H250" s="4" t="n"/>
+      <c r="I250" s="4" t="n"/>
+      <c r="J250" s="4" t="n"/>
+      <c r="K250" s="4" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="4" t="n"/>
@@ -2791,6 +3803,10 @@
       <c r="E251" s="4" t="n"/>
       <c r="F251" s="4" t="n"/>
       <c r="G251" s="4" t="n"/>
+      <c r="H251" s="4" t="n"/>
+      <c r="I251" s="4" t="n"/>
+      <c r="J251" s="4" t="n"/>
+      <c r="K251" s="4" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="4" t="n"/>
@@ -2800,6 +3816,10 @@
       <c r="E252" s="4" t="n"/>
       <c r="F252" s="4" t="n"/>
       <c r="G252" s="4" t="n"/>
+      <c r="H252" s="4" t="n"/>
+      <c r="I252" s="4" t="n"/>
+      <c r="J252" s="4" t="n"/>
+      <c r="K252" s="4" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="4" t="n"/>
@@ -2809,6 +3829,10 @@
       <c r="E253" s="4" t="n"/>
       <c r="F253" s="4" t="n"/>
       <c r="G253" s="4" t="n"/>
+      <c r="H253" s="4" t="n"/>
+      <c r="I253" s="4" t="n"/>
+      <c r="J253" s="4" t="n"/>
+      <c r="K253" s="4" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="4" t="n"/>
@@ -2818,6 +3842,10 @@
       <c r="E254" s="4" t="n"/>
       <c r="F254" s="4" t="n"/>
       <c r="G254" s="4" t="n"/>
+      <c r="H254" s="4" t="n"/>
+      <c r="I254" s="4" t="n"/>
+      <c r="J254" s="4" t="n"/>
+      <c r="K254" s="4" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="4" t="n"/>
@@ -2827,6 +3855,10 @@
       <c r="E255" s="4" t="n"/>
       <c r="F255" s="4" t="n"/>
       <c r="G255" s="4" t="n"/>
+      <c r="H255" s="4" t="n"/>
+      <c r="I255" s="4" t="n"/>
+      <c r="J255" s="4" t="n"/>
+      <c r="K255" s="4" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="4" t="n"/>
@@ -2836,6 +3868,10 @@
       <c r="E256" s="4" t="n"/>
       <c r="F256" s="4" t="n"/>
       <c r="G256" s="4" t="n"/>
+      <c r="H256" s="4" t="n"/>
+      <c r="I256" s="4" t="n"/>
+      <c r="J256" s="4" t="n"/>
+      <c r="K256" s="4" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="4" t="n"/>
@@ -2845,6 +3881,10 @@
       <c r="E257" s="4" t="n"/>
       <c r="F257" s="4" t="n"/>
       <c r="G257" s="4" t="n"/>
+      <c r="H257" s="4" t="n"/>
+      <c r="I257" s="4" t="n"/>
+      <c r="J257" s="4" t="n"/>
+      <c r="K257" s="4" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="4" t="n"/>
@@ -2854,6 +3894,10 @@
       <c r="E258" s="4" t="n"/>
       <c r="F258" s="4" t="n"/>
       <c r="G258" s="4" t="n"/>
+      <c r="H258" s="4" t="n"/>
+      <c r="I258" s="4" t="n"/>
+      <c r="J258" s="4" t="n"/>
+      <c r="K258" s="4" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="4" t="n"/>
@@ -2863,6 +3907,10 @@
       <c r="E259" s="4" t="n"/>
       <c r="F259" s="4" t="n"/>
       <c r="G259" s="4" t="n"/>
+      <c r="H259" s="4" t="n"/>
+      <c r="I259" s="4" t="n"/>
+      <c r="J259" s="4" t="n"/>
+      <c r="K259" s="4" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="4" t="n"/>
@@ -2872,6 +3920,10 @@
       <c r="E260" s="4" t="n"/>
       <c r="F260" s="4" t="n"/>
       <c r="G260" s="4" t="n"/>
+      <c r="H260" s="4" t="n"/>
+      <c r="I260" s="4" t="n"/>
+      <c r="J260" s="4" t="n"/>
+      <c r="K260" s="4" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="4" t="n"/>
@@ -2881,6 +3933,10 @@
       <c r="E261" s="4" t="n"/>
       <c r="F261" s="4" t="n"/>
       <c r="G261" s="4" t="n"/>
+      <c r="H261" s="4" t="n"/>
+      <c r="I261" s="4" t="n"/>
+      <c r="J261" s="4" t="n"/>
+      <c r="K261" s="4" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="4" t="n"/>
@@ -2890,6 +3946,10 @@
       <c r="E262" s="4" t="n"/>
       <c r="F262" s="4" t="n"/>
       <c r="G262" s="4" t="n"/>
+      <c r="H262" s="4" t="n"/>
+      <c r="I262" s="4" t="n"/>
+      <c r="J262" s="4" t="n"/>
+      <c r="K262" s="4" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="4" t="n"/>
@@ -2899,6 +3959,10 @@
       <c r="E263" s="4" t="n"/>
       <c r="F263" s="4" t="n"/>
       <c r="G263" s="4" t="n"/>
+      <c r="H263" s="4" t="n"/>
+      <c r="I263" s="4" t="n"/>
+      <c r="J263" s="4" t="n"/>
+      <c r="K263" s="4" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="4" t="n"/>
@@ -2908,6 +3972,10 @@
       <c r="E264" s="4" t="n"/>
       <c r="F264" s="4" t="n"/>
       <c r="G264" s="4" t="n"/>
+      <c r="H264" s="4" t="n"/>
+      <c r="I264" s="4" t="n"/>
+      <c r="J264" s="4" t="n"/>
+      <c r="K264" s="4" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="4" t="n"/>
@@ -2917,6 +3985,10 @@
       <c r="E265" s="4" t="n"/>
       <c r="F265" s="4" t="n"/>
       <c r="G265" s="4" t="n"/>
+      <c r="H265" s="4" t="n"/>
+      <c r="I265" s="4" t="n"/>
+      <c r="J265" s="4" t="n"/>
+      <c r="K265" s="4" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="4" t="n"/>
@@ -2926,6 +3998,10 @@
       <c r="E266" s="4" t="n"/>
       <c r="F266" s="4" t="n"/>
       <c r="G266" s="4" t="n"/>
+      <c r="H266" s="4" t="n"/>
+      <c r="I266" s="4" t="n"/>
+      <c r="J266" s="4" t="n"/>
+      <c r="K266" s="4" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="4" t="n"/>
@@ -2935,6 +4011,10 @@
       <c r="E267" s="4" t="n"/>
       <c r="F267" s="4" t="n"/>
       <c r="G267" s="4" t="n"/>
+      <c r="H267" s="4" t="n"/>
+      <c r="I267" s="4" t="n"/>
+      <c r="J267" s="4" t="n"/>
+      <c r="K267" s="4" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="4" t="n"/>
@@ -2944,6 +4024,10 @@
       <c r="E268" s="4" t="n"/>
       <c r="F268" s="4" t="n"/>
       <c r="G268" s="4" t="n"/>
+      <c r="H268" s="4" t="n"/>
+      <c r="I268" s="4" t="n"/>
+      <c r="J268" s="4" t="n"/>
+      <c r="K268" s="4" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="4" t="n"/>
@@ -2953,6 +4037,10 @@
       <c r="E269" s="4" t="n"/>
       <c r="F269" s="4" t="n"/>
       <c r="G269" s="4" t="n"/>
+      <c r="H269" s="4" t="n"/>
+      <c r="I269" s="4" t="n"/>
+      <c r="J269" s="4" t="n"/>
+      <c r="K269" s="4" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="4" t="n"/>
@@ -2962,6 +4050,10 @@
       <c r="E270" s="4" t="n"/>
       <c r="F270" s="4" t="n"/>
       <c r="G270" s="4" t="n"/>
+      <c r="H270" s="4" t="n"/>
+      <c r="I270" s="4" t="n"/>
+      <c r="J270" s="4" t="n"/>
+      <c r="K270" s="4" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="4" t="n"/>
@@ -2971,6 +4063,10 @@
       <c r="E271" s="4" t="n"/>
       <c r="F271" s="4" t="n"/>
       <c r="G271" s="4" t="n"/>
+      <c r="H271" s="4" t="n"/>
+      <c r="I271" s="4" t="n"/>
+      <c r="J271" s="4" t="n"/>
+      <c r="K271" s="4" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="4" t="n"/>
@@ -2980,6 +4076,10 @@
       <c r="E272" s="4" t="n"/>
       <c r="F272" s="4" t="n"/>
       <c r="G272" s="4" t="n"/>
+      <c r="H272" s="4" t="n"/>
+      <c r="I272" s="4" t="n"/>
+      <c r="J272" s="4" t="n"/>
+      <c r="K272" s="4" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="4" t="n"/>
@@ -2989,6 +4089,10 @@
       <c r="E273" s="4" t="n"/>
       <c r="F273" s="4" t="n"/>
       <c r="G273" s="4" t="n"/>
+      <c r="H273" s="4" t="n"/>
+      <c r="I273" s="4" t="n"/>
+      <c r="J273" s="4" t="n"/>
+      <c r="K273" s="4" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="4" t="n"/>
@@ -2998,6 +4102,10 @@
       <c r="E274" s="4" t="n"/>
       <c r="F274" s="4" t="n"/>
       <c r="G274" s="4" t="n"/>
+      <c r="H274" s="4" t="n"/>
+      <c r="I274" s="4" t="n"/>
+      <c r="J274" s="4" t="n"/>
+      <c r="K274" s="4" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="4" t="n"/>
@@ -3007,6 +4115,10 @@
       <c r="E275" s="4" t="n"/>
       <c r="F275" s="4" t="n"/>
       <c r="G275" s="4" t="n"/>
+      <c r="H275" s="4" t="n"/>
+      <c r="I275" s="4" t="n"/>
+      <c r="J275" s="4" t="n"/>
+      <c r="K275" s="4" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="4" t="n"/>
@@ -3016,6 +4128,10 @@
       <c r="E276" s="4" t="n"/>
       <c r="F276" s="4" t="n"/>
       <c r="G276" s="4" t="n"/>
+      <c r="H276" s="4" t="n"/>
+      <c r="I276" s="4" t="n"/>
+      <c r="J276" s="4" t="n"/>
+      <c r="K276" s="4" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="4" t="n"/>
@@ -3025,6 +4141,10 @@
       <c r="E277" s="4" t="n"/>
       <c r="F277" s="4" t="n"/>
       <c r="G277" s="4" t="n"/>
+      <c r="H277" s="4" t="n"/>
+      <c r="I277" s="4" t="n"/>
+      <c r="J277" s="4" t="n"/>
+      <c r="K277" s="4" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="4" t="n"/>
@@ -3034,6 +4154,10 @@
       <c r="E278" s="4" t="n"/>
       <c r="F278" s="4" t="n"/>
       <c r="G278" s="4" t="n"/>
+      <c r="H278" s="4" t="n"/>
+      <c r="I278" s="4" t="n"/>
+      <c r="J278" s="4" t="n"/>
+      <c r="K278" s="4" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="4" t="n"/>
@@ -3043,6 +4167,10 @@
       <c r="E279" s="4" t="n"/>
       <c r="F279" s="4" t="n"/>
       <c r="G279" s="4" t="n"/>
+      <c r="H279" s="4" t="n"/>
+      <c r="I279" s="4" t="n"/>
+      <c r="J279" s="4" t="n"/>
+      <c r="K279" s="4" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="4" t="n"/>
@@ -3052,6 +4180,10 @@
       <c r="E280" s="4" t="n"/>
       <c r="F280" s="4" t="n"/>
       <c r="G280" s="4" t="n"/>
+      <c r="H280" s="4" t="n"/>
+      <c r="I280" s="4" t="n"/>
+      <c r="J280" s="4" t="n"/>
+      <c r="K280" s="4" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="4" t="n"/>
@@ -3061,6 +4193,10 @@
       <c r="E281" s="4" t="n"/>
       <c r="F281" s="4" t="n"/>
       <c r="G281" s="4" t="n"/>
+      <c r="H281" s="4" t="n"/>
+      <c r="I281" s="4" t="n"/>
+      <c r="J281" s="4" t="n"/>
+      <c r="K281" s="4" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="4" t="n"/>
@@ -3070,6 +4206,10 @@
       <c r="E282" s="4" t="n"/>
       <c r="F282" s="4" t="n"/>
       <c r="G282" s="4" t="n"/>
+      <c r="H282" s="4" t="n"/>
+      <c r="I282" s="4" t="n"/>
+      <c r="J282" s="4" t="n"/>
+      <c r="K282" s="4" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="4" t="n"/>
@@ -3079,6 +4219,10 @@
       <c r="E283" s="4" t="n"/>
       <c r="F283" s="4" t="n"/>
       <c r="G283" s="4" t="n"/>
+      <c r="H283" s="4" t="n"/>
+      <c r="I283" s="4" t="n"/>
+      <c r="J283" s="4" t="n"/>
+      <c r="K283" s="4" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="4" t="n"/>
@@ -3088,6 +4232,10 @@
       <c r="E284" s="4" t="n"/>
       <c r="F284" s="4" t="n"/>
       <c r="G284" s="4" t="n"/>
+      <c r="H284" s="4" t="n"/>
+      <c r="I284" s="4" t="n"/>
+      <c r="J284" s="4" t="n"/>
+      <c r="K284" s="4" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="4" t="n"/>
@@ -3097,6 +4245,10 @@
       <c r="E285" s="4" t="n"/>
       <c r="F285" s="4" t="n"/>
       <c r="G285" s="4" t="n"/>
+      <c r="H285" s="4" t="n"/>
+      <c r="I285" s="4" t="n"/>
+      <c r="J285" s="4" t="n"/>
+      <c r="K285" s="4" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="4" t="n"/>
@@ -3106,6 +4258,10 @@
       <c r="E286" s="4" t="n"/>
       <c r="F286" s="4" t="n"/>
       <c r="G286" s="4" t="n"/>
+      <c r="H286" s="4" t="n"/>
+      <c r="I286" s="4" t="n"/>
+      <c r="J286" s="4" t="n"/>
+      <c r="K286" s="4" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="4" t="n"/>
@@ -3115,6 +4271,10 @@
       <c r="E287" s="4" t="n"/>
       <c r="F287" s="4" t="n"/>
       <c r="G287" s="4" t="n"/>
+      <c r="H287" s="4" t="n"/>
+      <c r="I287" s="4" t="n"/>
+      <c r="J287" s="4" t="n"/>
+      <c r="K287" s="4" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="4" t="n"/>
@@ -3124,6 +4284,10 @@
       <c r="E288" s="4" t="n"/>
       <c r="F288" s="4" t="n"/>
       <c r="G288" s="4" t="n"/>
+      <c r="H288" s="4" t="n"/>
+      <c r="I288" s="4" t="n"/>
+      <c r="J288" s="4" t="n"/>
+      <c r="K288" s="4" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="4" t="n"/>
@@ -3133,6 +4297,10 @@
       <c r="E289" s="4" t="n"/>
       <c r="F289" s="4" t="n"/>
       <c r="G289" s="4" t="n"/>
+      <c r="H289" s="4" t="n"/>
+      <c r="I289" s="4" t="n"/>
+      <c r="J289" s="4" t="n"/>
+      <c r="K289" s="4" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="4" t="n"/>
@@ -3142,6 +4310,10 @@
       <c r="E290" s="4" t="n"/>
       <c r="F290" s="4" t="n"/>
       <c r="G290" s="4" t="n"/>
+      <c r="H290" s="4" t="n"/>
+      <c r="I290" s="4" t="n"/>
+      <c r="J290" s="4" t="n"/>
+      <c r="K290" s="4" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="4" t="n"/>
@@ -3151,6 +4323,10 @@
       <c r="E291" s="4" t="n"/>
       <c r="F291" s="4" t="n"/>
       <c r="G291" s="4" t="n"/>
+      <c r="H291" s="4" t="n"/>
+      <c r="I291" s="4" t="n"/>
+      <c r="J291" s="4" t="n"/>
+      <c r="K291" s="4" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="4" t="n"/>
@@ -3160,6 +4336,10 @@
       <c r="E292" s="4" t="n"/>
       <c r="F292" s="4" t="n"/>
       <c r="G292" s="4" t="n"/>
+      <c r="H292" s="4" t="n"/>
+      <c r="I292" s="4" t="n"/>
+      <c r="J292" s="4" t="n"/>
+      <c r="K292" s="4" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="4" t="n"/>
@@ -3169,6 +4349,10 @@
       <c r="E293" s="4" t="n"/>
       <c r="F293" s="4" t="n"/>
       <c r="G293" s="4" t="n"/>
+      <c r="H293" s="4" t="n"/>
+      <c r="I293" s="4" t="n"/>
+      <c r="J293" s="4" t="n"/>
+      <c r="K293" s="4" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="4" t="n"/>
@@ -3178,6 +4362,10 @@
       <c r="E294" s="4" t="n"/>
       <c r="F294" s="4" t="n"/>
       <c r="G294" s="4" t="n"/>
+      <c r="H294" s="4" t="n"/>
+      <c r="I294" s="4" t="n"/>
+      <c r="J294" s="4" t="n"/>
+      <c r="K294" s="4" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="4" t="n"/>
@@ -3187,6 +4375,10 @@
       <c r="E295" s="4" t="n"/>
       <c r="F295" s="4" t="n"/>
       <c r="G295" s="4" t="n"/>
+      <c r="H295" s="4" t="n"/>
+      <c r="I295" s="4" t="n"/>
+      <c r="J295" s="4" t="n"/>
+      <c r="K295" s="4" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="4" t="n"/>
@@ -3196,6 +4388,10 @@
       <c r="E296" s="4" t="n"/>
       <c r="F296" s="4" t="n"/>
       <c r="G296" s="4" t="n"/>
+      <c r="H296" s="4" t="n"/>
+      <c r="I296" s="4" t="n"/>
+      <c r="J296" s="4" t="n"/>
+      <c r="K296" s="4" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="4" t="n"/>
@@ -3205,6 +4401,10 @@
       <c r="E297" s="4" t="n"/>
       <c r="F297" s="4" t="n"/>
       <c r="G297" s="4" t="n"/>
+      <c r="H297" s="4" t="n"/>
+      <c r="I297" s="4" t="n"/>
+      <c r="J297" s="4" t="n"/>
+      <c r="K297" s="4" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="4" t="n"/>
@@ -3214,6 +4414,10 @@
       <c r="E298" s="4" t="n"/>
       <c r="F298" s="4" t="n"/>
       <c r="G298" s="4" t="n"/>
+      <c r="H298" s="4" t="n"/>
+      <c r="I298" s="4" t="n"/>
+      <c r="J298" s="4" t="n"/>
+      <c r="K298" s="4" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="4" t="n"/>
@@ -3223,6 +4427,10 @@
       <c r="E299" s="4" t="n"/>
       <c r="F299" s="4" t="n"/>
       <c r="G299" s="4" t="n"/>
+      <c r="H299" s="4" t="n"/>
+      <c r="I299" s="4" t="n"/>
+      <c r="J299" s="4" t="n"/>
+      <c r="K299" s="4" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="4" t="n"/>
@@ -3232,6 +4440,10 @@
       <c r="E300" s="4" t="n"/>
       <c r="F300" s="4" t="n"/>
       <c r="G300" s="4" t="n"/>
+      <c r="H300" s="4" t="n"/>
+      <c r="I300" s="4" t="n"/>
+      <c r="J300" s="4" t="n"/>
+      <c r="K300" s="4" t="n"/>
     </row>
     <row r="301">
       <c r="A301" s="4" t="n"/>
@@ -3241,6 +4453,10 @@
       <c r="E301" s="4" t="n"/>
       <c r="F301" s="4" t="n"/>
       <c r="G301" s="4" t="n"/>
+      <c r="H301" s="4" t="n"/>
+      <c r="I301" s="4" t="n"/>
+      <c r="J301" s="4" t="n"/>
+      <c r="K301" s="4" t="n"/>
     </row>
     <row r="302">
       <c r="A302" s="4" t="n"/>
@@ -3250,6 +4466,10 @@
       <c r="E302" s="4" t="n"/>
       <c r="F302" s="4" t="n"/>
       <c r="G302" s="4" t="n"/>
+      <c r="H302" s="4" t="n"/>
+      <c r="I302" s="4" t="n"/>
+      <c r="J302" s="4" t="n"/>
+      <c r="K302" s="4" t="n"/>
     </row>
     <row r="303">
       <c r="A303" s="4" t="n"/>
@@ -3259,11 +4479,15 @@
       <c r="E303" s="4" t="n"/>
       <c r="F303" s="4" t="n"/>
       <c r="G303" s="4" t="n"/>
+      <c r="H303" s="4" t="n"/>
+      <c r="I303" s="4" t="n"/>
+      <c r="J303" s="4" t="n"/>
+      <c r="K303" s="4" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="B4:B304" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Not a valid type" error="Pick one of: franchise, centre, school, individual" promptTitle="Customer type" prompt="franchise / centre / school / individual" type="list">
@@ -3280,7 +4504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3288,8 +4512,12 @@
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -3327,10 +4555,30 @@
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>address</t>
+          <t>address1</t>
         </is>
       </c>
       <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>address2</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>city</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>postcode</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="K3" s="6" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -3354,8 +4602,24 @@
       </c>
       <c r="D4" s="7" t="inlineStr"/>
       <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Street / building.</t>
+        </is>
+      </c>
       <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>Town or city.</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="inlineStr"/>
+      <c r="J4" s="7" t="inlineStr">
+        <is>
+          <t>Blank means United Kingdom.</t>
+        </is>
+      </c>
+      <c r="K4" s="7" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -3385,12 +4649,28 @@
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>26 Haslucks Green Road, Solihull B90 2EL</t>
+          <t>The Exchange</t>
         </is>
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>Original centre</t>
+          <t>26 Haslucks Green Road</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>Solihull</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>B90 2EL</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr"/>
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>Invoices as Robocode Shirley</t>
         </is>
       </c>
     </row>
@@ -3422,6 +4702,18 @@
       </c>
       <c r="F6" s="8" t="inlineStr"/>
       <c r="G6" s="8" t="inlineStr"/>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>Leicester</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="inlineStr"/>
+      <c r="J6" s="8" t="inlineStr"/>
+      <c r="K6" s="8" t="inlineStr">
+        <is>
+          <t>Name only - no "Robocode" prefix</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
@@ -3445,8 +4737,24 @@
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr"/>
-      <c r="F7" s="8" t="inlineStr"/>
-      <c r="G7" s="8" t="inlineStr">
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>Woodthorpe Road</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr"/>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>Birmingham</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>B14 6EQ</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="inlineStr"/>
+      <c r="K7" s="8" t="inlineStr">
         <is>
           <t>Wednesday club</t>
         </is>
@@ -3478,8 +4786,24 @@
           <t>07700 900000</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr"/>
-      <c r="G8" s="8" t="inlineStr">
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>14 Beech Road</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr"/>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>Solihull</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>B91 1AA</t>
+        </is>
+      </c>
+      <c r="J8" s="8" t="inlineStr"/>
+      <c r="K8" s="8" t="inlineStr">
         <is>
           <t>Bought C1 outright</t>
         </is>
@@ -3487,7 +4811,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>